<commit_message>
fix: resubir template ContHumedad C566-25 sheet2 INFORME corregido
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/ContHumedad ASTM C566-25/1-INF.-N-000-26-AG20-CH-V08.xlsx
+++ b/app/templates/informes/Informes agregado/ContHumedad ASTM C566-25/1-INF.-N-000-26-AG20-CH-V08.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.2 Informe agregados\INFORME ACREDITADO-E ISO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\ContHumedad ASTM C566-25\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C094092C-5E03-42EE-926E-A33189E14D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A470AA5-8957-4A64-A792-123F7432E7F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="723" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="96" r:id="rId1"/>
@@ -3215,22 +3215,63 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -3240,10 +3281,6 @@
       <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
@@ -3269,50 +3306,28 @@
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="8" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="180" fontId="14" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -3354,24 +3369,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3414,30 +3411,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="19" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="176" fontId="2" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="4" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -3518,6 +3491,30 @@
     <xf numFmtId="2" fontId="7" fillId="2" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="19" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="10" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="12" xfId="3" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3537,6 +3534,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -4891,7 +4891,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -4950,7 +4950,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="datos de ecuacion del anillo"/>
@@ -5069,7 +5069,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -5120,7 +5120,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -5172,7 +5172,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink5.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -5204,7 +5204,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink6.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -5909,20 +5909,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1272CFCF-C297-4FBF-B59A-4BAC3921853B}">
   <dimension ref="A1:Q49"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" customWidth="1"/>
+    <col min="1" max="1" width="1.88671875" customWidth="1"/>
     <col min="2" max="2" width="3" customWidth="1"/>
-    <col min="5" max="5" width="17.42578125" customWidth="1"/>
-    <col min="6" max="6" width="5.28515625" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" customWidth="1"/>
-    <col min="8" max="8" width="3.28515625" customWidth="1"/>
-    <col min="9" max="9" width="5.7109375" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" customWidth="1"/>
-    <col min="11" max="11" width="10.28515625" customWidth="1"/>
-    <col min="12" max="12" width="1.5703125" customWidth="1"/>
-    <col min="13" max="13" width="5.28515625" customWidth="1"/>
-    <col min="14" max="14" width="14.42578125" customWidth="1"/>
+    <col min="5" max="5" width="17.44140625" customWidth="1"/>
+    <col min="6" max="6" width="5.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" customWidth="1"/>
+    <col min="8" max="8" width="3.33203125" customWidth="1"/>
+    <col min="9" max="9" width="5.6640625" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" customWidth="1"/>
+    <col min="11" max="11" width="10.33203125" customWidth="1"/>
+    <col min="12" max="12" width="1.5546875" customWidth="1"/>
+    <col min="13" max="13" width="5.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
@@ -6001,7 +6001,7 @@
       </c>
       <c r="Q4" s="377"/>
     </row>
-    <row r="5" spans="1:17" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="290"/>
       <c r="B5" s="291"/>
       <c r="C5" s="291"/>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="Q5" s="377"/>
     </row>
-    <row r="6" spans="1:17" ht="15.95" customHeight="1" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:17" ht="15.9" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A6" s="293"/>
       <c r="B6" s="293"/>
       <c r="C6" s="293"/>
@@ -6039,51 +6039,51 @@
       <c r="P6" s="378"/>
       <c r="Q6" s="379"/>
     </row>
-    <row r="7" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="414" t="s">
+    <row r="7" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="392" t="s">
         <v>0</v>
       </c>
-      <c r="B7" s="414"/>
-      <c r="C7" s="414"/>
-      <c r="D7" s="414"/>
-      <c r="E7" s="414"/>
-      <c r="F7" s="414"/>
-      <c r="G7" s="414"/>
-      <c r="H7" s="414"/>
-      <c r="I7" s="414"/>
-      <c r="J7" s="414"/>
-      <c r="K7" s="414"/>
-      <c r="L7" s="414"/>
-      <c r="M7" s="414"/>
-      <c r="N7" s="414"/>
+      <c r="B7" s="392"/>
+      <c r="C7" s="392"/>
+      <c r="D7" s="392"/>
+      <c r="E7" s="392"/>
+      <c r="F7" s="392"/>
+      <c r="G7" s="392"/>
+      <c r="H7" s="392"/>
+      <c r="I7" s="392"/>
+      <c r="J7" s="392"/>
+      <c r="K7" s="392"/>
+      <c r="L7" s="392"/>
+      <c r="M7" s="392"/>
+      <c r="N7" s="392"/>
       <c r="P7" s="380" t="s">
         <v>158</v>
       </c>
       <c r="Q7" s="379"/>
     </row>
-    <row r="8" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="415" t="s">
+    <row r="8" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="393" t="s">
         <v>162</v>
       </c>
-      <c r="B8" s="415"/>
-      <c r="C8" s="415"/>
-      <c r="D8" s="415"/>
-      <c r="E8" s="415"/>
-      <c r="F8" s="415"/>
-      <c r="G8" s="415"/>
-      <c r="H8" s="415"/>
-      <c r="I8" s="415"/>
-      <c r="J8" s="415"/>
-      <c r="K8" s="415"/>
-      <c r="L8" s="415"/>
-      <c r="M8" s="415"/>
-      <c r="N8" s="415"/>
+      <c r="B8" s="393"/>
+      <c r="C8" s="393"/>
+      <c r="D8" s="393"/>
+      <c r="E8" s="393"/>
+      <c r="F8" s="393"/>
+      <c r="G8" s="393"/>
+      <c r="H8" s="393"/>
+      <c r="I8" s="393"/>
+      <c r="J8" s="393"/>
+      <c r="K8" s="393"/>
+      <c r="L8" s="393"/>
+      <c r="M8" s="393"/>
+      <c r="N8" s="393"/>
       <c r="P8" s="380" t="s">
         <v>198</v>
       </c>
       <c r="Q8" s="381"/>
     </row>
-    <row r="9" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="294"/>
       <c r="B9" s="294"/>
       <c r="C9" s="294"/>
@@ -6103,65 +6103,65 @@
       </c>
       <c r="Q9" s="379"/>
     </row>
-    <row r="10" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="294"/>
       <c r="B10" s="294"/>
       <c r="C10" s="294"/>
       <c r="D10" s="294"/>
-      <c r="E10" s="416" t="s">
+      <c r="E10" s="394" t="s">
         <v>163</v>
       </c>
-      <c r="F10" s="416"/>
+      <c r="F10" s="394"/>
       <c r="G10" s="295" t="s">
         <v>164</v>
       </c>
-      <c r="H10" s="416" t="s">
+      <c r="H10" s="394" t="s">
         <v>165</v>
       </c>
-      <c r="I10" s="416"/>
-      <c r="J10" s="416"/>
-      <c r="K10" s="416" t="s">
+      <c r="I10" s="394"/>
+      <c r="J10" s="394"/>
+      <c r="K10" s="394" t="s">
         <v>166</v>
       </c>
-      <c r="L10" s="416"/>
-      <c r="M10" s="416"/>
+      <c r="L10" s="394"/>
+      <c r="M10" s="394"/>
       <c r="N10" s="294"/>
       <c r="P10" s="378"/>
       <c r="Q10" s="379"/>
     </row>
-    <row r="11" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="294"/>
       <c r="B11" s="294"/>
       <c r="C11" s="294"/>
       <c r="D11" s="294"/>
-      <c r="E11" s="413"/>
-      <c r="F11" s="413"/>
+      <c r="E11" s="391"/>
+      <c r="F11" s="391"/>
       <c r="G11" s="296"/>
-      <c r="H11" s="413"/>
-      <c r="I11" s="413"/>
-      <c r="J11" s="413"/>
-      <c r="K11" s="413"/>
-      <c r="L11" s="413"/>
-      <c r="M11" s="413"/>
+      <c r="H11" s="391"/>
+      <c r="I11" s="391"/>
+      <c r="J11" s="391"/>
+      <c r="K11" s="391"/>
+      <c r="L11" s="391"/>
+      <c r="M11" s="391"/>
       <c r="N11" s="294"/>
       <c r="P11" s="380" t="s">
         <v>13</v>
       </c>
       <c r="Q11" s="379"/>
     </row>
-    <row r="12" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="288"/>
-      <c r="B12" s="392"/>
-      <c r="C12" s="392"/>
-      <c r="D12" s="392"/>
-      <c r="E12" s="392"/>
-      <c r="F12" s="392"/>
-      <c r="G12" s="392"/>
-      <c r="H12" s="392"/>
-      <c r="I12" s="392"/>
-      <c r="J12" s="392"/>
-      <c r="K12" s="392"/>
-      <c r="L12" s="392"/>
+      <c r="B12" s="396"/>
+      <c r="C12" s="396"/>
+      <c r="D12" s="396"/>
+      <c r="E12" s="396"/>
+      <c r="F12" s="396"/>
+      <c r="G12" s="396"/>
+      <c r="H12" s="396"/>
+      <c r="I12" s="396"/>
+      <c r="J12" s="396"/>
+      <c r="K12" s="396"/>
+      <c r="L12" s="396"/>
       <c r="M12" s="297"/>
       <c r="N12" s="298"/>
       <c r="P12" s="380" t="s">
@@ -6169,7 +6169,7 @@
       </c>
       <c r="Q12" s="381"/>
     </row>
-    <row r="13" spans="1:17" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:17" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="299"/>
       <c r="B13" s="297"/>
       <c r="C13" s="297"/>
@@ -6189,49 +6189,49 @@
       </c>
       <c r="Q13" s="381"/>
     </row>
-    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="406" t="s">
+    <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="397" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="407"/>
-      <c r="C14" s="407"/>
-      <c r="D14" s="407"/>
-      <c r="E14" s="407"/>
-      <c r="F14" s="407"/>
-      <c r="G14" s="407"/>
-      <c r="H14" s="407"/>
-      <c r="I14" s="407"/>
-      <c r="J14" s="407"/>
-      <c r="K14" s="407"/>
-      <c r="L14" s="407"/>
-      <c r="M14" s="407"/>
-      <c r="N14" s="408"/>
+      <c r="B14" s="398"/>
+      <c r="C14" s="398"/>
+      <c r="D14" s="398"/>
+      <c r="E14" s="398"/>
+      <c r="F14" s="398"/>
+      <c r="G14" s="398"/>
+      <c r="H14" s="398"/>
+      <c r="I14" s="398"/>
+      <c r="J14" s="398"/>
+      <c r="K14" s="398"/>
+      <c r="L14" s="398"/>
+      <c r="M14" s="398"/>
+      <c r="N14" s="399"/>
       <c r="P14" s="378"/>
       <c r="Q14" s="379"/>
     </row>
-    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="409" t="s">
+    <row r="15" spans="1:17" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="400" t="s">
         <v>161</v>
       </c>
-      <c r="B15" s="410"/>
-      <c r="C15" s="410"/>
-      <c r="D15" s="410"/>
-      <c r="E15" s="410"/>
-      <c r="F15" s="410"/>
-      <c r="G15" s="410"/>
-      <c r="H15" s="410"/>
-      <c r="I15" s="410"/>
-      <c r="J15" s="410"/>
-      <c r="K15" s="410"/>
-      <c r="L15" s="410"/>
-      <c r="M15" s="410"/>
-      <c r="N15" s="411"/>
+      <c r="B15" s="401"/>
+      <c r="C15" s="401"/>
+      <c r="D15" s="401"/>
+      <c r="E15" s="401"/>
+      <c r="F15" s="401"/>
+      <c r="G15" s="401"/>
+      <c r="H15" s="401"/>
+      <c r="I15" s="401"/>
+      <c r="J15" s="401"/>
+      <c r="K15" s="401"/>
+      <c r="L15" s="401"/>
+      <c r="M15" s="401"/>
+      <c r="N15" s="402"/>
       <c r="P15" s="380" t="s">
         <v>200</v>
       </c>
       <c r="Q15" s="382"/>
     </row>
-    <row r="16" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="303"/>
       <c r="B16" s="304"/>
       <c r="C16" s="304"/>
@@ -6262,8 +6262,8 @@
       <c r="H17" s="309"/>
       <c r="I17" s="309"/>
       <c r="J17" s="309"/>
-      <c r="K17" s="412"/>
-      <c r="L17" s="412"/>
+      <c r="K17" s="403"/>
+      <c r="L17" s="403"/>
       <c r="M17" s="310"/>
       <c r="N17" s="311"/>
       <c r="P17" s="380" t="s">
@@ -6273,19 +6273,19 @@
     </row>
     <row r="18" spans="1:17" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="312"/>
-      <c r="B18" s="399" t="s">
+      <c r="B18" s="395" t="s">
         <v>19</v>
       </c>
-      <c r="C18" s="399"/>
-      <c r="D18" s="399"/>
-      <c r="E18" s="399"/>
+      <c r="C18" s="395"/>
+      <c r="D18" s="395"/>
+      <c r="E18" s="395"/>
       <c r="F18" s="313" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="399" t="s">
+      <c r="G18" s="395" t="s">
         <v>167</v>
       </c>
-      <c r="H18" s="399"/>
+      <c r="H18" s="395"/>
       <c r="I18" s="314"/>
       <c r="J18" s="288"/>
       <c r="K18" s="315"/>
@@ -6293,7 +6293,7 @@
       <c r="M18" s="315"/>
       <c r="N18" s="316"/>
     </row>
-    <row r="19" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="317"/>
       <c r="B19" s="318">
         <v>1</v>
@@ -6306,8 +6306,8 @@
       <c r="F19" s="322" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="399"/>
-      <c r="H19" s="399"/>
+      <c r="G19" s="395"/>
+      <c r="H19" s="395"/>
       <c r="I19" s="323"/>
       <c r="J19" s="324"/>
       <c r="K19" s="324"/>
@@ -6315,7 +6315,7 @@
       <c r="M19" s="325"/>
       <c r="N19" s="326"/>
     </row>
-    <row r="20" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="317"/>
       <c r="B20" s="327">
         <v>2</v>
@@ -6328,8 +6328,8 @@
       <c r="F20" s="331" t="s">
         <v>23</v>
       </c>
-      <c r="G20" s="399"/>
-      <c r="H20" s="399"/>
+      <c r="G20" s="395"/>
+      <c r="H20" s="395"/>
       <c r="I20" s="323"/>
       <c r="J20" s="332"/>
       <c r="K20" s="333"/>
@@ -6337,7 +6337,7 @@
       <c r="M20" s="334"/>
       <c r="N20" s="335"/>
     </row>
-    <row r="21" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="317"/>
       <c r="B21" s="336">
         <v>3</v>
@@ -6350,8 +6350,8 @@
       <c r="F21" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="G21" s="399"/>
-      <c r="H21" s="399"/>
+      <c r="G21" s="395"/>
+      <c r="H21" s="395"/>
       <c r="I21" s="323"/>
       <c r="J21" s="341"/>
       <c r="K21" s="333"/>
@@ -6359,7 +6359,7 @@
       <c r="M21" s="342"/>
       <c r="N21" s="343"/>
     </row>
-    <row r="22" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="317"/>
       <c r="B22" s="336">
         <v>4</v>
@@ -6372,8 +6372,8 @@
       <c r="F22" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="G22" s="399"/>
-      <c r="H22" s="399"/>
+      <c r="G22" s="395"/>
+      <c r="H22" s="395"/>
       <c r="I22" s="323"/>
       <c r="J22" s="332"/>
       <c r="K22" s="332"/>
@@ -6381,7 +6381,7 @@
       <c r="M22" s="342"/>
       <c r="N22" s="343"/>
     </row>
-    <row r="23" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="317"/>
       <c r="B23" s="336">
         <v>5</v>
@@ -6394,8 +6394,8 @@
       <c r="F23" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="G23" s="399"/>
-      <c r="H23" s="399"/>
+      <c r="G23" s="395"/>
+      <c r="H23" s="395"/>
       <c r="I23" s="323"/>
       <c r="J23" s="332"/>
       <c r="K23" s="332"/>
@@ -6403,7 +6403,7 @@
       <c r="M23" s="342"/>
       <c r="N23" s="343"/>
     </row>
-    <row r="24" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="317"/>
       <c r="B24" s="336">
         <v>6</v>
@@ -6416,8 +6416,8 @@
       <c r="F24" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="G24" s="399"/>
-      <c r="H24" s="399"/>
+      <c r="G24" s="395"/>
+      <c r="H24" s="395"/>
       <c r="I24" s="323"/>
       <c r="J24" s="288"/>
       <c r="K24" s="344"/>
@@ -6425,7 +6425,7 @@
       <c r="M24" s="342"/>
       <c r="N24" s="343"/>
     </row>
-    <row r="25" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="345"/>
       <c r="B25" s="336">
         <v>7</v>
@@ -6438,8 +6438,8 @@
       <c r="F25" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="G25" s="399"/>
-      <c r="H25" s="399"/>
+      <c r="G25" s="395"/>
+      <c r="H25" s="395"/>
       <c r="I25" s="323"/>
       <c r="J25" s="288"/>
       <c r="K25" s="342"/>
@@ -6447,7 +6447,7 @@
       <c r="M25" s="342"/>
       <c r="N25" s="343"/>
     </row>
-    <row r="26" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="317"/>
       <c r="B26" s="336">
         <v>8</v>
@@ -6460,8 +6460,8 @@
       <c r="F26" s="340" t="s">
         <v>26</v>
       </c>
-      <c r="G26" s="399"/>
-      <c r="H26" s="399"/>
+      <c r="G26" s="395"/>
+      <c r="H26" s="395"/>
       <c r="I26" s="323"/>
       <c r="J26" s="288"/>
       <c r="K26" s="346"/>
@@ -6469,7 +6469,7 @@
       <c r="M26" s="342"/>
       <c r="N26" s="343"/>
     </row>
-    <row r="27" spans="1:17" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" ht="23.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="317"/>
       <c r="B27" s="336">
         <v>9</v>
@@ -6482,16 +6482,16 @@
       <c r="F27" s="340" t="s">
         <v>32</v>
       </c>
-      <c r="G27" s="399"/>
-      <c r="H27" s="399"/>
-      <c r="I27" s="400" t="s">
+      <c r="G27" s="395"/>
+      <c r="H27" s="395"/>
+      <c r="I27" s="410" t="s">
         <v>173</v>
       </c>
-      <c r="J27" s="400"/>
-      <c r="K27" s="400"/>
-      <c r="L27" s="400"/>
-      <c r="M27" s="400"/>
-      <c r="N27" s="401"/>
+      <c r="J27" s="410"/>
+      <c r="K27" s="410"/>
+      <c r="L27" s="410"/>
+      <c r="M27" s="410"/>
+      <c r="N27" s="411"/>
     </row>
     <row r="28" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="317"/>
@@ -6504,12 +6504,12 @@
       <c r="F28" s="288"/>
       <c r="G28" s="288"/>
       <c r="H28" s="288"/>
-      <c r="I28" s="400"/>
-      <c r="J28" s="400"/>
-      <c r="K28" s="400"/>
-      <c r="L28" s="400"/>
-      <c r="M28" s="400"/>
-      <c r="N28" s="401"/>
+      <c r="I28" s="410"/>
+      <c r="J28" s="410"/>
+      <c r="K28" s="410"/>
+      <c r="L28" s="410"/>
+      <c r="M28" s="410"/>
+      <c r="N28" s="411"/>
     </row>
     <row r="29" spans="1:17" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="317"/>
@@ -6537,18 +6537,18 @@
       <c r="C30" s="351"/>
       <c r="D30" s="351"/>
       <c r="E30" s="351"/>
-      <c r="F30" s="402"/>
-      <c r="G30" s="402"/>
+      <c r="F30" s="412"/>
+      <c r="G30" s="412"/>
       <c r="H30" s="288"/>
-      <c r="I30" s="403" t="s">
+      <c r="I30" s="413" t="s">
         <v>177</v>
       </c>
-      <c r="J30" s="404"/>
-      <c r="K30" s="403" t="s">
+      <c r="J30" s="414"/>
+      <c r="K30" s="413" t="s">
         <v>178</v>
       </c>
-      <c r="L30" s="405"/>
-      <c r="M30" s="404"/>
+      <c r="L30" s="415"/>
+      <c r="M30" s="414"/>
       <c r="N30" s="349"/>
     </row>
     <row r="31" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6559,36 +6559,36 @@
       <c r="C31" s="351"/>
       <c r="D31" s="351"/>
       <c r="E31" s="351"/>
-      <c r="F31" s="391"/>
-      <c r="G31" s="391"/>
+      <c r="F31" s="406"/>
+      <c r="G31" s="406"/>
       <c r="H31" s="288"/>
       <c r="I31" s="352" t="s">
         <v>180</v>
       </c>
       <c r="J31" s="353"/>
-      <c r="K31" s="396"/>
-      <c r="L31" s="397"/>
-      <c r="M31" s="398"/>
+      <c r="K31" s="407"/>
+      <c r="L31" s="408"/>
+      <c r="M31" s="409"/>
       <c r="N31" s="349"/>
     </row>
     <row r="32" spans="1:17" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="317"/>
-      <c r="B32" s="394" t="s">
+      <c r="B32" s="404" t="s">
         <v>181</v>
       </c>
-      <c r="C32" s="394"/>
-      <c r="D32" s="394"/>
-      <c r="E32" s="395"/>
-      <c r="F32" s="391"/>
-      <c r="G32" s="391"/>
+      <c r="C32" s="404"/>
+      <c r="D32" s="404"/>
+      <c r="E32" s="405"/>
+      <c r="F32" s="406"/>
+      <c r="G32" s="406"/>
       <c r="H32" s="288"/>
       <c r="I32" s="352" t="s">
         <v>182</v>
       </c>
       <c r="J32" s="353"/>
-      <c r="K32" s="396"/>
-      <c r="L32" s="397"/>
-      <c r="M32" s="398"/>
+      <c r="K32" s="407"/>
+      <c r="L32" s="408"/>
+      <c r="M32" s="409"/>
       <c r="N32" s="349"/>
     </row>
     <row r="33" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -6599,8 +6599,8 @@
       <c r="C33" s="351"/>
       <c r="D33" s="351"/>
       <c r="E33" s="351"/>
-      <c r="F33" s="391"/>
-      <c r="G33" s="391"/>
+      <c r="F33" s="406"/>
+      <c r="G33" s="406"/>
       <c r="H33" s="288"/>
       <c r="I33" s="288"/>
       <c r="J33" s="288"/>
@@ -6699,7 +6699,7 @@
       <c r="M38" s="288"/>
       <c r="N38" s="288"/>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" s="368"/>
       <c r="B39" s="369"/>
       <c r="C39" s="369"/>
@@ -6715,7 +6715,7 @@
       <c r="M39" s="342"/>
       <c r="N39" s="342"/>
     </row>
-    <row r="40" spans="1:14" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="370"/>
       <c r="B40" s="369"/>
       <c r="C40" s="369"/>
@@ -6731,7 +6731,7 @@
       <c r="M40" s="342"/>
       <c r="N40" s="342"/>
     </row>
-    <row r="41" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="370"/>
       <c r="B41" s="369"/>
       <c r="C41" s="369"/>
@@ -6747,7 +6747,7 @@
       <c r="M41" s="342"/>
       <c r="N41" s="342"/>
     </row>
-    <row r="42" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="370"/>
       <c r="B42" s="369"/>
       <c r="C42" s="369"/>
@@ -6779,7 +6779,7 @@
       <c r="M43" s="342"/>
       <c r="N43" s="342"/>
     </row>
-    <row r="44" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="368"/>
       <c r="B44" s="369"/>
       <c r="C44" s="369"/>
@@ -6797,21 +6797,21 @@
     </row>
     <row r="45" spans="1:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="288"/>
-      <c r="B45" s="392"/>
-      <c r="C45" s="392"/>
-      <c r="D45" s="392"/>
-      <c r="E45" s="392"/>
-      <c r="F45" s="392"/>
-      <c r="G45" s="392"/>
-      <c r="H45" s="392"/>
-      <c r="I45" s="392"/>
-      <c r="J45" s="392"/>
-      <c r="K45" s="392"/>
-      <c r="L45" s="392"/>
+      <c r="B45" s="396"/>
+      <c r="C45" s="396"/>
+      <c r="D45" s="396"/>
+      <c r="E45" s="396"/>
+      <c r="F45" s="396"/>
+      <c r="G45" s="396"/>
+      <c r="H45" s="396"/>
+      <c r="I45" s="396"/>
+      <c r="J45" s="396"/>
+      <c r="K45" s="396"/>
+      <c r="L45" s="396"/>
       <c r="M45" s="297"/>
       <c r="N45" s="342"/>
     </row>
-    <row r="46" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="372" t="s">
         <v>38</v>
       </c>
@@ -6865,23 +6865,23 @@
       <c r="M48" s="288"/>
       <c r="N48" s="288"/>
     </row>
-    <row r="49" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="393" t="s">
+    <row r="49" spans="1:14" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="416" t="s">
         <v>191</v>
       </c>
-      <c r="B49" s="393"/>
-      <c r="C49" s="393"/>
-      <c r="D49" s="393"/>
-      <c r="E49" s="393"/>
-      <c r="F49" s="393"/>
-      <c r="G49" s="393"/>
-      <c r="H49" s="393"/>
-      <c r="I49" s="393"/>
-      <c r="J49" s="393"/>
-      <c r="K49" s="393"/>
-      <c r="L49" s="393"/>
-      <c r="M49" s="393"/>
-      <c r="N49" s="393"/>
+      <c r="B49" s="416"/>
+      <c r="C49" s="416"/>
+      <c r="D49" s="416"/>
+      <c r="E49" s="416"/>
+      <c r="F49" s="416"/>
+      <c r="G49" s="416"/>
+      <c r="H49" s="416"/>
+      <c r="I49" s="416"/>
+      <c r="J49" s="416"/>
+      <c r="K49" s="416"/>
+      <c r="L49" s="416"/>
+      <c r="M49" s="416"/>
+      <c r="N49" s="416"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="w1vl+vEjAtd8PhMkrP3wy2fn0tyF73b+R9UYCJzZUsz+xBZyT1FXTpLlkkyENiLui5lLbEiRmQlWsxzqarVT9A==" saltValue="kGFq1o2+4sMRy0cFC5vQJA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
@@ -6890,26 +6890,11 @@
     <protectedRange sqref="D45 D12" name="Rango3_3_1_1_1_1_1_2_1_2"/>
   </protectedRanges>
   <mergeCells count="39">
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="H11:J11"/>
-    <mergeCell ref="K11:M11"/>
-    <mergeCell ref="A7:N7"/>
-    <mergeCell ref="A8:N8"/>
-    <mergeCell ref="E10:F10"/>
-    <mergeCell ref="H10:J10"/>
-    <mergeCell ref="K10:M10"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="F12:I12"/>
-    <mergeCell ref="J12:L12"/>
-    <mergeCell ref="A14:N14"/>
-    <mergeCell ref="A15:N15"/>
-    <mergeCell ref="K17:L17"/>
-    <mergeCell ref="B18:E18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="J45:L45"/>
+    <mergeCell ref="A49:N49"/>
     <mergeCell ref="B32:E32"/>
     <mergeCell ref="F32:G32"/>
     <mergeCell ref="K32:M32"/>
@@ -6924,11 +6909,26 @@
     <mergeCell ref="K30:M30"/>
     <mergeCell ref="F31:G31"/>
     <mergeCell ref="K31:M31"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="B45:E45"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="J45:L45"/>
-    <mergeCell ref="A49:N49"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="F12:I12"/>
+    <mergeCell ref="J12:L12"/>
+    <mergeCell ref="A14:N14"/>
+    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="K17:L17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="H11:J11"/>
+    <mergeCell ref="K11:M11"/>
+    <mergeCell ref="A7:N7"/>
+    <mergeCell ref="A8:N8"/>
+    <mergeCell ref="E10:F10"/>
+    <mergeCell ref="H10:J10"/>
+    <mergeCell ref="K10:M10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
@@ -6940,27 +6940,27 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Hoja2"/>
   <dimension ref="A1:P54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="1.85546875" style="23" customWidth="1"/>
+    <col min="1" max="1" width="1.88671875" style="23" customWidth="1"/>
     <col min="2" max="2" width="9" style="23" customWidth="1"/>
-    <col min="3" max="3" width="2.85546875" style="23" customWidth="1"/>
-    <col min="4" max="4" width="5.140625" style="23" customWidth="1"/>
-    <col min="5" max="5" width="2.28515625" style="23" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="23" customWidth="1"/>
-    <col min="7" max="7" width="9.7109375" style="23" customWidth="1"/>
+    <col min="3" max="3" width="2.88671875" style="23" customWidth="1"/>
+    <col min="4" max="4" width="5.109375" style="23" customWidth="1"/>
+    <col min="5" max="5" width="2.33203125" style="23" customWidth="1"/>
+    <col min="6" max="6" width="10.88671875" style="23" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" style="23" customWidth="1"/>
     <col min="8" max="8" width="8" style="23" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" style="23" customWidth="1"/>
-    <col min="10" max="10" width="9.7109375" style="23" customWidth="1"/>
-    <col min="11" max="11" width="9.28515625" style="23" customWidth="1"/>
-    <col min="12" max="12" width="13.28515625" style="23" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" style="23" customWidth="1"/>
+    <col min="10" max="10" width="9.6640625" style="23" customWidth="1"/>
+    <col min="11" max="11" width="9.33203125" style="23" customWidth="1"/>
+    <col min="12" max="12" width="13.33203125" style="23" customWidth="1"/>
     <col min="13" max="13" width="1" style="23" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" style="23" customWidth="1"/>
-    <col min="15" max="16" width="6.42578125" style="23" customWidth="1"/>
-    <col min="17" max="16384" width="10.28515625" style="23"/>
+    <col min="14" max="14" width="13.5546875" style="23" customWidth="1"/>
+    <col min="15" max="16" width="6.44140625" style="23" customWidth="1"/>
+    <col min="17" max="16384" width="10.33203125" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="34"/>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -6976,44 +6976,44 @@
       <c r="M1" s="34"/>
       <c r="N1" s="34"/>
     </row>
-    <row r="2" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="417" t="s">
+    <row r="2" spans="1:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="491" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="417"/>
-      <c r="C2" s="417"/>
-      <c r="D2" s="417"/>
-      <c r="E2" s="417"/>
-      <c r="F2" s="417"/>
-      <c r="G2" s="417"/>
-      <c r="H2" s="417"/>
-      <c r="I2" s="417"/>
-      <c r="J2" s="417"/>
-      <c r="K2" s="417"/>
-      <c r="L2" s="417"/>
-      <c r="M2" s="417"/>
-      <c r="N2" s="417"/>
-    </row>
-    <row r="3" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="419">
+      <c r="B2" s="491"/>
+      <c r="C2" s="491"/>
+      <c r="D2" s="491"/>
+      <c r="E2" s="491"/>
+      <c r="F2" s="491"/>
+      <c r="G2" s="491"/>
+      <c r="H2" s="491"/>
+      <c r="I2" s="491"/>
+      <c r="J2" s="491"/>
+      <c r="K2" s="491"/>
+      <c r="L2" s="491"/>
+      <c r="M2" s="491"/>
+      <c r="N2" s="491"/>
+    </row>
+    <row r="3" spans="1:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="424">
         <v>0</v>
       </c>
-      <c r="B3" s="419"/>
-      <c r="C3" s="419"/>
-      <c r="D3" s="419"/>
-      <c r="E3" s="419"/>
-      <c r="F3" s="419"/>
-      <c r="G3" s="419"/>
-      <c r="H3" s="419"/>
-      <c r="I3" s="419"/>
-      <c r="J3" s="419"/>
-      <c r="K3" s="419"/>
-      <c r="L3" s="419"/>
-      <c r="M3" s="419"/>
-      <c r="N3" s="419"/>
-    </row>
-    <row r="4" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="424"/>
+      <c r="C3" s="424"/>
+      <c r="D3" s="424"/>
+      <c r="E3" s="424"/>
+      <c r="F3" s="424"/>
+      <c r="G3" s="424"/>
+      <c r="H3" s="424"/>
+      <c r="I3" s="424"/>
+      <c r="J3" s="424"/>
+      <c r="K3" s="424"/>
+      <c r="L3" s="424"/>
+      <c r="M3" s="424"/>
+      <c r="N3" s="424"/>
+    </row>
+    <row r="4" spans="1:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="5" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="181" t="s">
         <v>1</v>
       </c>
@@ -7021,17 +7021,17 @@
       <c r="C5" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="430">
+      <c r="D5" s="435">
         <f>+FORMATO!Q2</f>
         <v>0</v>
       </c>
-      <c r="E5" s="430"/>
-      <c r="F5" s="430"/>
-      <c r="G5" s="430"/>
-      <c r="H5" s="430"/>
-      <c r="I5" s="430"/>
-      <c r="J5" s="430"/>
-      <c r="K5" s="430"/>
+      <c r="E5" s="435"/>
+      <c r="F5" s="435"/>
+      <c r="G5" s="435"/>
+      <c r="H5" s="435"/>
+      <c r="I5" s="435"/>
+      <c r="J5" s="435"/>
+      <c r="K5" s="435"/>
       <c r="L5" s="179" t="s">
         <v>3</v>
       </c>
@@ -7042,7 +7042,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="181" t="s">
         <v>5</v>
       </c>
@@ -7050,17 +7050,17 @@
       <c r="C6" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="430">
+      <c r="D6" s="435">
         <f>+FORMATO!Q3</f>
         <v>0</v>
       </c>
-      <c r="E6" s="430"/>
-      <c r="F6" s="430"/>
-      <c r="G6" s="430"/>
-      <c r="H6" s="430"/>
-      <c r="I6" s="430"/>
-      <c r="J6" s="430"/>
-      <c r="K6" s="430"/>
+      <c r="E6" s="435"/>
+      <c r="F6" s="435"/>
+      <c r="G6" s="435"/>
+      <c r="H6" s="435"/>
+      <c r="I6" s="435"/>
+      <c r="J6" s="435"/>
+      <c r="K6" s="435"/>
       <c r="L6" s="390" t="s">
         <v>158</v>
       </c>
@@ -7074,7 +7074,7 @@
       <c r="O6" s="24"/>
       <c r="P6" s="24"/>
     </row>
-    <row r="7" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="181" t="s">
         <v>6</v>
       </c>
@@ -7082,17 +7082,17 @@
       <c r="C7" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="430">
+      <c r="D7" s="435">
         <f>+FORMATO!Q4</f>
         <v>0</v>
       </c>
-      <c r="E7" s="430"/>
-      <c r="F7" s="430"/>
-      <c r="G7" s="430"/>
-      <c r="H7" s="430"/>
-      <c r="I7" s="430"/>
-      <c r="J7" s="430"/>
-      <c r="K7" s="430"/>
+      <c r="E7" s="435"/>
+      <c r="F7" s="435"/>
+      <c r="G7" s="435"/>
+      <c r="H7" s="435"/>
+      <c r="I7" s="435"/>
+      <c r="J7" s="435"/>
+      <c r="K7" s="435"/>
       <c r="L7" s="179" t="s">
         <v>199</v>
       </c>
@@ -7106,7 +7106,7 @@
       <c r="O7" s="24"/>
       <c r="P7" s="24"/>
     </row>
-    <row r="8" spans="1:16" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="181" t="s">
         <v>7</v>
       </c>
@@ -7114,17 +7114,17 @@
       <c r="C8" s="66" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="430">
+      <c r="D8" s="435">
         <f>+FORMATO!Q5</f>
         <v>0</v>
       </c>
-      <c r="E8" s="430"/>
-      <c r="F8" s="430"/>
-      <c r="G8" s="430"/>
-      <c r="H8" s="430"/>
-      <c r="I8" s="430"/>
-      <c r="J8" s="430"/>
-      <c r="K8" s="430"/>
+      <c r="E8" s="435"/>
+      <c r="F8" s="435"/>
+      <c r="G8" s="435"/>
+      <c r="H8" s="435"/>
+      <c r="I8" s="435"/>
+      <c r="J8" s="435"/>
+      <c r="K8" s="435"/>
       <c r="L8" s="390" t="s">
         <v>208</v>
       </c>
@@ -7138,7 +7138,7 @@
       <c r="O8" s="24"/>
       <c r="P8" s="24"/>
     </row>
-    <row r="9" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="176" t="s">
         <v>8</v>
       </c>
@@ -7158,47 +7158,47 @@
       <c r="O9" s="24"/>
       <c r="P9" s="24"/>
     </row>
-    <row r="10" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="422" t="s">
+    <row r="10" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="427" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="423"/>
-      <c r="C10" s="423"/>
-      <c r="D10" s="423"/>
-      <c r="E10" s="423"/>
-      <c r="F10" s="423"/>
-      <c r="G10" s="423"/>
-      <c r="H10" s="423"/>
-      <c r="I10" s="423"/>
-      <c r="J10" s="423"/>
-      <c r="K10" s="423"/>
-      <c r="L10" s="423"/>
-      <c r="M10" s="423"/>
-      <c r="N10" s="424"/>
+      <c r="B10" s="428"/>
+      <c r="C10" s="428"/>
+      <c r="D10" s="428"/>
+      <c r="E10" s="428"/>
+      <c r="F10" s="428"/>
+      <c r="G10" s="428"/>
+      <c r="H10" s="428"/>
+      <c r="I10" s="428"/>
+      <c r="J10" s="428"/>
+      <c r="K10" s="428"/>
+      <c r="L10" s="428"/>
+      <c r="M10" s="428"/>
+      <c r="N10" s="429"/>
       <c r="O10" s="24"/>
       <c r="P10" s="24"/>
     </row>
-    <row r="11" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="425" t="s">
+    <row r="11" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="430" t="s">
         <v>160</v>
       </c>
-      <c r="B11" s="426"/>
-      <c r="C11" s="426"/>
-      <c r="D11" s="426"/>
-      <c r="E11" s="426"/>
-      <c r="F11" s="426"/>
-      <c r="G11" s="426"/>
-      <c r="H11" s="426"/>
-      <c r="I11" s="426"/>
-      <c r="J11" s="426"/>
-      <c r="K11" s="426"/>
-      <c r="L11" s="426"/>
-      <c r="M11" s="426"/>
-      <c r="N11" s="427"/>
+      <c r="B11" s="431"/>
+      <c r="C11" s="431"/>
+      <c r="D11" s="431"/>
+      <c r="E11" s="431"/>
+      <c r="F11" s="431"/>
+      <c r="G11" s="431"/>
+      <c r="H11" s="431"/>
+      <c r="I11" s="431"/>
+      <c r="J11" s="431"/>
+      <c r="K11" s="431"/>
+      <c r="L11" s="431"/>
+      <c r="M11" s="431"/>
+      <c r="N11" s="432"/>
       <c r="O11" s="24"/>
       <c r="P11" s="24"/>
     </row>
-    <row r="12" spans="1:16" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="37"/>
       <c r="B12" s="38"/>
       <c r="C12" s="38"/>
@@ -7216,7 +7216,7 @@
       <c r="O12" s="24"/>
       <c r="P12" s="24"/>
     </row>
-    <row r="13" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="39" t="s">
         <v>11</v>
       </c>
@@ -7235,7 +7235,7 @@
       <c r="N13" s="20"/>
       <c r="P13" s="24"/>
     </row>
-    <row r="14" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="40" t="s">
         <v>12</v>
       </c>
@@ -7265,7 +7265,7 @@
       </c>
       <c r="P14" s="24"/>
     </row>
-    <row r="15" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="40" t="s">
         <v>14</v>
       </c>
@@ -7295,7 +7295,7 @@
       </c>
       <c r="P15" s="24"/>
     </row>
-    <row r="16" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="40" t="s">
         <v>157</v>
       </c>
@@ -7305,11 +7305,11 @@
       <c r="E16" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="F16" s="429">
+      <c r="F16" s="434">
         <f>+FORMATO!Q17</f>
         <v>0</v>
       </c>
-      <c r="G16" s="429"/>
+      <c r="G16" s="434"/>
       <c r="H16" s="22"/>
       <c r="I16" s="22"/>
       <c r="J16" s="22"/>
@@ -7330,7 +7330,7 @@
       </c>
       <c r="P16" s="24"/>
     </row>
-    <row r="17" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="40" t="s">
         <v>17</v>
       </c>
@@ -7353,7 +7353,7 @@
       <c r="N17" s="21"/>
       <c r="P17" s="24"/>
     </row>
-    <row r="18" spans="1:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="41"/>
       <c r="B18" s="103"/>
       <c r="C18" s="103"/>
@@ -7370,36 +7370,36 @@
       <c r="N18" s="30"/>
       <c r="P18" s="24"/>
     </row>
-    <row r="19" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="44"/>
       <c r="B19" s="212"/>
       <c r="C19" s="212"/>
       <c r="D19" s="212"/>
-      <c r="E19" s="420"/>
-      <c r="F19" s="420"/>
+      <c r="E19" s="425"/>
+      <c r="F19" s="425"/>
       <c r="G19" s="212"/>
       <c r="H19" s="212"/>
       <c r="I19" s="212"/>
       <c r="J19" s="212"/>
       <c r="K19" s="212"/>
-      <c r="L19" s="420"/>
-      <c r="M19" s="420"/>
+      <c r="L19" s="425"/>
+      <c r="M19" s="425"/>
       <c r="N19" s="45"/>
       <c r="O19" s="24"/>
       <c r="P19" s="31"/>
     </row>
-    <row r="20" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="44"/>
       <c r="B20" s="212"/>
       <c r="C20" s="212"/>
       <c r="D20" s="212"/>
       <c r="E20" s="212"/>
-      <c r="F20" s="428" t="s">
+      <c r="F20" s="433" t="s">
         <v>19</v>
       </c>
-      <c r="G20" s="428"/>
-      <c r="H20" s="428"/>
-      <c r="I20" s="428"/>
+      <c r="G20" s="433"/>
+      <c r="H20" s="433"/>
+      <c r="I20" s="433"/>
       <c r="J20" s="213" t="s">
         <v>20</v>
       </c>
@@ -7412,18 +7412,18 @@
       <c r="O20" s="24"/>
       <c r="P20" s="31"/>
     </row>
-    <row r="21" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="46"/>
       <c r="B21" s="35"/>
       <c r="C21" s="35"/>
       <c r="D21" s="35"/>
       <c r="E21" s="35"/>
-      <c r="F21" s="418" t="s">
+      <c r="F21" s="419" t="s">
         <v>22</v>
       </c>
-      <c r="G21" s="418"/>
-      <c r="H21" s="418"/>
-      <c r="I21" s="418"/>
+      <c r="G21" s="419"/>
+      <c r="H21" s="419"/>
+      <c r="I21" s="419"/>
       <c r="J21" s="47" t="s">
         <v>23</v>
       </c>
@@ -7431,24 +7431,24 @@
         <f>+'Datos ensayo'!D13</f>
         <v>1</v>
       </c>
-      <c r="L21" s="421"/>
-      <c r="M21" s="421"/>
+      <c r="L21" s="426"/>
+      <c r="M21" s="426"/>
       <c r="N21" s="49"/>
       <c r="O21" s="24"/>
       <c r="P21" s="32"/>
     </row>
-    <row r="22" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="46"/>
       <c r="B22" s="35"/>
       <c r="C22" s="35"/>
       <c r="D22" s="35"/>
       <c r="E22" s="35"/>
-      <c r="F22" s="418" t="s">
+      <c r="F22" s="419" t="s">
         <v>24</v>
       </c>
-      <c r="G22" s="418"/>
-      <c r="H22" s="418"/>
-      <c r="I22" s="418"/>
+      <c r="G22" s="419"/>
+      <c r="H22" s="419"/>
+      <c r="I22" s="419"/>
       <c r="J22" s="47" t="s">
         <v>23</v>
       </c>
@@ -7456,24 +7456,24 @@
         <f>+'Datos ensayo'!D14</f>
         <v>0</v>
       </c>
-      <c r="L22" s="421"/>
-      <c r="M22" s="421"/>
+      <c r="L22" s="426"/>
+      <c r="M22" s="426"/>
       <c r="N22" s="49"/>
       <c r="O22" s="24"/>
       <c r="P22" s="32"/>
     </row>
-    <row r="23" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="46"/>
       <c r="B23" s="35"/>
       <c r="C23" s="35"/>
       <c r="D23" s="35"/>
       <c r="E23" s="35"/>
-      <c r="F23" s="418" t="s">
+      <c r="F23" s="419" t="s">
         <v>25</v>
       </c>
-      <c r="G23" s="418"/>
-      <c r="H23" s="418"/>
-      <c r="I23" s="418"/>
+      <c r="G23" s="419"/>
+      <c r="H23" s="419"/>
+      <c r="I23" s="419"/>
       <c r="J23" s="47" t="s">
         <v>26</v>
       </c>
@@ -7481,24 +7481,24 @@
         <f>+'Datos ensayo'!E15</f>
         <v>0</v>
       </c>
-      <c r="L23" s="432"/>
-      <c r="M23" s="432"/>
+      <c r="L23" s="418"/>
+      <c r="M23" s="418"/>
       <c r="N23" s="52"/>
       <c r="O23" s="33"/>
       <c r="P23" s="32"/>
     </row>
-    <row r="24" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="46"/>
       <c r="B24" s="35"/>
       <c r="C24" s="35"/>
       <c r="D24" s="35"/>
       <c r="E24" s="35"/>
-      <c r="F24" s="418" t="s">
+      <c r="F24" s="419" t="s">
         <v>27</v>
       </c>
-      <c r="G24" s="418"/>
-      <c r="H24" s="418"/>
-      <c r="I24" s="418"/>
+      <c r="G24" s="419"/>
+      <c r="H24" s="419"/>
+      <c r="I24" s="419"/>
       <c r="J24" s="47" t="s">
         <v>26</v>
       </c>
@@ -7512,18 +7512,18 @@
       <c r="O24" s="24"/>
       <c r="P24" s="24"/>
     </row>
-    <row r="25" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="46"/>
       <c r="B25" s="35"/>
       <c r="C25" s="35"/>
       <c r="D25" s="35"/>
       <c r="E25" s="35"/>
-      <c r="F25" s="418" t="s">
+      <c r="F25" s="419" t="s">
         <v>28</v>
       </c>
-      <c r="G25" s="418"/>
-      <c r="H25" s="418"/>
-      <c r="I25" s="418"/>
+      <c r="G25" s="419"/>
+      <c r="H25" s="419"/>
+      <c r="I25" s="419"/>
       <c r="J25" s="47" t="s">
         <v>26</v>
       </c>
@@ -7537,18 +7537,18 @@
       <c r="O25" s="24"/>
       <c r="P25" s="24"/>
     </row>
-    <row r="26" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="46"/>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
       <c r="D26" s="35"/>
       <c r="E26" s="35"/>
-      <c r="F26" s="418" t="s">
+      <c r="F26" s="419" t="s">
         <v>29</v>
       </c>
-      <c r="G26" s="418"/>
-      <c r="H26" s="418"/>
-      <c r="I26" s="418"/>
+      <c r="G26" s="419"/>
+      <c r="H26" s="419"/>
+      <c r="I26" s="419"/>
       <c r="J26" s="47" t="s">
         <v>26</v>
       </c>
@@ -7562,18 +7562,18 @@
       <c r="O26" s="24"/>
       <c r="P26" s="24"/>
     </row>
-    <row r="27" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="46"/>
       <c r="B27" s="35"/>
       <c r="C27" s="35"/>
       <c r="D27" s="35"/>
       <c r="E27" s="35"/>
-      <c r="F27" s="418" t="s">
+      <c r="F27" s="419" t="s">
         <v>30</v>
       </c>
-      <c r="G27" s="418"/>
-      <c r="H27" s="418"/>
-      <c r="I27" s="418"/>
+      <c r="G27" s="419"/>
+      <c r="H27" s="419"/>
+      <c r="I27" s="419"/>
       <c r="J27" s="47" t="s">
         <v>26</v>
       </c>
@@ -7587,18 +7587,18 @@
       <c r="O27" s="24"/>
       <c r="P27" s="24"/>
     </row>
-    <row r="28" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="46"/>
       <c r="B28" s="35"/>
       <c r="C28" s="35"/>
       <c r="D28" s="35"/>
       <c r="E28" s="35"/>
-      <c r="F28" s="418" t="s">
+      <c r="F28" s="419" t="s">
         <v>31</v>
       </c>
-      <c r="G28" s="418"/>
-      <c r="H28" s="418"/>
-      <c r="I28" s="418"/>
+      <c r="G28" s="419"/>
+      <c r="H28" s="419"/>
+      <c r="I28" s="419"/>
       <c r="J28" s="47" t="s">
         <v>32</v>
       </c>
@@ -7612,7 +7612,7 @@
       <c r="O28" s="24"/>
       <c r="P28" s="24"/>
     </row>
-    <row r="29" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:16" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="56"/>
       <c r="B29" s="59"/>
       <c r="C29" s="59"/>
@@ -7630,16 +7630,16 @@
       <c r="O29" s="24"/>
       <c r="P29" s="24"/>
     </row>
-    <row r="30" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="35"/>
       <c r="B30" s="35"/>
       <c r="C30" s="35"/>
       <c r="D30" s="35"/>
       <c r="E30" s="35"/>
-      <c r="F30" s="433"/>
-      <c r="G30" s="433"/>
-      <c r="H30" s="433"/>
-      <c r="I30" s="433"/>
+      <c r="F30" s="420"/>
+      <c r="G30" s="420"/>
+      <c r="H30" s="420"/>
+      <c r="I30" s="420"/>
       <c r="J30" s="61"/>
       <c r="K30" s="62"/>
       <c r="L30" s="53"/>
@@ -7648,7 +7648,7 @@
       <c r="O30" s="24"/>
       <c r="P30" s="24"/>
     </row>
-    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="165" t="s">
         <v>33</v>
       </c>
@@ -7668,7 +7668,7 @@
       <c r="O31" s="24"/>
       <c r="P31" s="24"/>
     </row>
-    <row r="32" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="172" t="s">
         <v>34</v>
       </c>
@@ -7689,7 +7689,7 @@
       <c r="O32" s="24"/>
       <c r="P32" s="24"/>
     </row>
-    <row r="33" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="172"/>
       <c r="B33" s="170"/>
       <c r="C33" s="170"/>
@@ -7705,7 +7705,7 @@
       <c r="O33" s="24"/>
       <c r="P33" s="24"/>
     </row>
-    <row r="34" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:16" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="165" t="s">
         <v>152</v>
       </c>
@@ -7723,7 +7723,7 @@
       <c r="O34" s="24"/>
       <c r="P34" s="24"/>
     </row>
-    <row r="35" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="170" t="s">
         <v>154</v>
       </c>
@@ -7744,7 +7744,7 @@
       <c r="O35" s="24"/>
       <c r="P35" s="24"/>
     </row>
-    <row r="36" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="170" t="s">
         <v>153</v>
       </c>
@@ -7767,7 +7767,7 @@
       <c r="O36" s="24"/>
       <c r="P36" s="24"/>
     </row>
-    <row r="37" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="170"/>
       <c r="B37" s="35"/>
       <c r="C37" s="35"/>
@@ -7785,7 +7785,7 @@
       <c r="O37" s="24"/>
       <c r="P37" s="24"/>
     </row>
-    <row r="38" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="165" t="s">
         <v>35</v>
       </c>
@@ -7803,97 +7803,97 @@
       <c r="O38" s="24"/>
       <c r="P38" s="24"/>
     </row>
-    <row r="39" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="436" t="s">
+    <row r="39" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="423" t="s">
         <v>209</v>
       </c>
-      <c r="B39" s="436"/>
-      <c r="C39" s="436"/>
-      <c r="D39" s="436"/>
-      <c r="E39" s="436"/>
-      <c r="F39" s="436"/>
-      <c r="G39" s="436"/>
-      <c r="H39" s="436"/>
-      <c r="I39" s="436"/>
-      <c r="J39" s="436"/>
-      <c r="K39" s="436"/>
-      <c r="L39" s="436"/>
-      <c r="M39" s="436"/>
-      <c r="N39" s="436"/>
+      <c r="B39" s="423"/>
+      <c r="C39" s="423"/>
+      <c r="D39" s="423"/>
+      <c r="E39" s="423"/>
+      <c r="F39" s="423"/>
+      <c r="G39" s="423"/>
+      <c r="H39" s="423"/>
+      <c r="I39" s="423"/>
+      <c r="J39" s="423"/>
+      <c r="K39" s="423"/>
+      <c r="L39" s="423"/>
+      <c r="M39" s="423"/>
+      <c r="N39" s="423"/>
       <c r="O39" s="24"/>
       <c r="P39" s="24"/>
     </row>
-    <row r="40" spans="1:16" ht="28.9" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="434" t="s">
+    <row r="40" spans="1:16" ht="28.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="421" t="s">
         <v>210</v>
       </c>
-      <c r="B40" s="434"/>
-      <c r="C40" s="434"/>
-      <c r="D40" s="434"/>
-      <c r="E40" s="434"/>
-      <c r="F40" s="434"/>
-      <c r="G40" s="434"/>
-      <c r="H40" s="434"/>
-      <c r="I40" s="434"/>
-      <c r="J40" s="434"/>
-      <c r="K40" s="434"/>
-      <c r="L40" s="434"/>
-      <c r="M40" s="434"/>
-      <c r="N40" s="434"/>
-    </row>
-    <row r="41" spans="1:16" ht="19.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="434" t="s">
+      <c r="B40" s="421"/>
+      <c r="C40" s="421"/>
+      <c r="D40" s="421"/>
+      <c r="E40" s="421"/>
+      <c r="F40" s="421"/>
+      <c r="G40" s="421"/>
+      <c r="H40" s="421"/>
+      <c r="I40" s="421"/>
+      <c r="J40" s="421"/>
+      <c r="K40" s="421"/>
+      <c r="L40" s="421"/>
+      <c r="M40" s="421"/>
+      <c r="N40" s="421"/>
+    </row>
+    <row r="41" spans="1:16" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="421" t="s">
         <v>211</v>
       </c>
-      <c r="B41" s="434"/>
-      <c r="C41" s="434"/>
-      <c r="D41" s="434"/>
-      <c r="E41" s="434"/>
-      <c r="F41" s="434"/>
-      <c r="G41" s="434"/>
-      <c r="H41" s="434"/>
-      <c r="I41" s="434"/>
-      <c r="J41" s="434"/>
-      <c r="K41" s="434"/>
-      <c r="L41" s="434"/>
-      <c r="M41" s="434"/>
-      <c r="N41" s="434"/>
-    </row>
-    <row r="42" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="434" t="s">
+      <c r="B41" s="421"/>
+      <c r="C41" s="421"/>
+      <c r="D41" s="421"/>
+      <c r="E41" s="421"/>
+      <c r="F41" s="421"/>
+      <c r="G41" s="421"/>
+      <c r="H41" s="421"/>
+      <c r="I41" s="421"/>
+      <c r="J41" s="421"/>
+      <c r="K41" s="421"/>
+      <c r="L41" s="421"/>
+      <c r="M41" s="421"/>
+      <c r="N41" s="421"/>
+    </row>
+    <row r="42" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="421" t="s">
         <v>212</v>
       </c>
-      <c r="B42" s="434"/>
-      <c r="C42" s="434"/>
-      <c r="D42" s="434"/>
-      <c r="E42" s="434"/>
-      <c r="F42" s="434"/>
-      <c r="G42" s="434"/>
-      <c r="H42" s="434"/>
-      <c r="I42" s="434"/>
-      <c r="J42" s="434"/>
-      <c r="K42" s="434"/>
-      <c r="L42" s="434"/>
-      <c r="M42" s="434"/>
-      <c r="N42" s="434"/>
-    </row>
-    <row r="43" spans="1:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="435" t="s">
+      <c r="B42" s="421"/>
+      <c r="C42" s="421"/>
+      <c r="D42" s="421"/>
+      <c r="E42" s="421"/>
+      <c r="F42" s="421"/>
+      <c r="G42" s="421"/>
+      <c r="H42" s="421"/>
+      <c r="I42" s="421"/>
+      <c r="J42" s="421"/>
+      <c r="K42" s="421"/>
+      <c r="L42" s="421"/>
+      <c r="M42" s="421"/>
+      <c r="N42" s="421"/>
+    </row>
+    <row r="43" spans="1:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="422" t="s">
         <v>213</v>
       </c>
-      <c r="B43" s="435"/>
-      <c r="C43" s="435"/>
-      <c r="D43" s="435"/>
-      <c r="E43" s="435"/>
-      <c r="F43" s="435"/>
-      <c r="G43" s="435"/>
-      <c r="H43" s="435"/>
-      <c r="I43" s="435"/>
-      <c r="J43" s="435"/>
-      <c r="K43" s="435"/>
-      <c r="L43" s="435"/>
-      <c r="M43" s="435"/>
-      <c r="N43" s="435"/>
+      <c r="B43" s="422"/>
+      <c r="C43" s="422"/>
+      <c r="D43" s="422"/>
+      <c r="E43" s="422"/>
+      <c r="F43" s="422"/>
+      <c r="G43" s="422"/>
+      <c r="H43" s="422"/>
+      <c r="I43" s="422"/>
+      <c r="J43" s="422"/>
+      <c r="K43" s="422"/>
+      <c r="L43" s="422"/>
+      <c r="M43" s="422"/>
+      <c r="N43" s="422"/>
     </row>
     <row r="44" spans="1:16" ht="9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B44" s="76"/>
@@ -7926,7 +7926,7 @@
       <c r="M45" s="182"/>
       <c r="N45" s="182"/>
     </row>
-    <row r="46" spans="1:16" ht="60.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:16" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D46" s="35"/>
       <c r="E46" s="35"/>
       <c r="F46" s="35"/>
@@ -7935,7 +7935,7 @@
       <c r="I46" s="35"/>
       <c r="J46" s="35"/>
     </row>
-    <row r="47" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D47" s="35"/>
       <c r="E47" s="35"/>
       <c r="F47" s="35"/>
@@ -7943,12 +7943,12 @@
       <c r="H47" s="35"/>
       <c r="I47" s="35"/>
       <c r="J47" s="35"/>
-      <c r="K47" s="431"/>
-      <c r="L47" s="431"/>
-      <c r="M47" s="431"/>
-      <c r="N47" s="431"/>
-    </row>
-    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K47" s="417"/>
+      <c r="L47" s="417"/>
+      <c r="M47" s="417"/>
+      <c r="N47" s="417"/>
+    </row>
+    <row r="48" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="64"/>
       <c r="D48" s="35"/>
       <c r="E48" s="35"/>
@@ -7958,7 +7958,7 @@
       <c r="I48" s="35"/>
       <c r="J48" s="35"/>
     </row>
-    <row r="49" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="64" t="s">
         <v>38</v>
       </c>
@@ -7970,7 +7970,7 @@
       <c r="I49" s="35"/>
       <c r="J49" s="35"/>
     </row>
-    <row r="50" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="64" t="s">
         <v>214</v>
       </c>
@@ -7983,12 +7983,12 @@
       <c r="H50" s="35"/>
       <c r="I50" s="35"/>
       <c r="J50" s="35"/>
-      <c r="K50" s="431" t="s">
+      <c r="K50" s="417" t="s">
         <v>37</v>
       </c>
-      <c r="L50" s="431"/>
-      <c r="M50" s="431"/>
-      <c r="N50" s="431"/>
+      <c r="L50" s="417"/>
+      <c r="M50" s="417"/>
+      <c r="N50" s="417"/>
     </row>
     <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="64"/>
@@ -8005,7 +8005,7 @@
       <c r="M51" s="35"/>
       <c r="N51" s="35"/>
     </row>
-    <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="64"/>
       <c r="B52" s="64"/>
       <c r="C52" s="64"/>
@@ -8021,7 +8021,7 @@
       <c r="M52" s="35"/>
       <c r="N52" s="35"/>
     </row>
-    <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="64"/>
       <c r="B53" s="64"/>
       <c r="C53" s="64"/>
@@ -8033,7 +8033,7 @@
       <c r="I53" s="35"/>
       <c r="J53" s="35"/>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="35"/>
       <c r="B54" s="35"/>
       <c r="C54" s="35"/>
@@ -8050,26 +8050,10 @@
       <c r="N54" s="35"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="x3BFs7mdqsnx2M2YraLXdNNVH6g+kcDZ8pY0xUnh6hitaQ+nfHjxr/q5PX8J+Rtr0w7Rg4o0Ew4zZN+snR+eMg==" saltValue="LAzxgemv8QgIKifmvtEmtQ==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <protectedRanges>
     <protectedRange sqref="F12 F9" name="Rango3_3_1_1_1_1_1_1_1_1"/>
   </protectedRanges>
   <mergeCells count="31">
-    <mergeCell ref="K50:N50"/>
-    <mergeCell ref="L23:M23"/>
-    <mergeCell ref="F23:I23"/>
-    <mergeCell ref="K47:N47"/>
-    <mergeCell ref="F28:I28"/>
-    <mergeCell ref="F24:I24"/>
-    <mergeCell ref="F30:I30"/>
-    <mergeCell ref="F25:I25"/>
-    <mergeCell ref="F26:I26"/>
-    <mergeCell ref="F27:I27"/>
-    <mergeCell ref="A41:N41"/>
-    <mergeCell ref="A43:N43"/>
-    <mergeCell ref="A42:N42"/>
-    <mergeCell ref="A39:N39"/>
-    <mergeCell ref="A40:N40"/>
     <mergeCell ref="A2:N2"/>
     <mergeCell ref="F21:I21"/>
     <mergeCell ref="F22:I22"/>
@@ -8086,6 +8070,21 @@
     <mergeCell ref="D8:K8"/>
     <mergeCell ref="D7:K7"/>
     <mergeCell ref="D6:K6"/>
+    <mergeCell ref="K50:N50"/>
+    <mergeCell ref="L23:M23"/>
+    <mergeCell ref="F23:I23"/>
+    <mergeCell ref="K47:N47"/>
+    <mergeCell ref="F28:I28"/>
+    <mergeCell ref="F24:I24"/>
+    <mergeCell ref="F30:I30"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="F26:I26"/>
+    <mergeCell ref="F27:I27"/>
+    <mergeCell ref="A41:N41"/>
+    <mergeCell ref="A43:N43"/>
+    <mergeCell ref="A42:N42"/>
+    <mergeCell ref="A39:N39"/>
+    <mergeCell ref="A40:N40"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations disablePrompts="1" count="1">
@@ -8110,21 +8109,21 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P42"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.28515625" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.33203125" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" style="23" customWidth="1"/>
-    <col min="2" max="2" width="40.140625" style="23" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" style="23"/>
-    <col min="4" max="4" width="10.28515625" style="23" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" style="23" customWidth="1"/>
-    <col min="6" max="6" width="12.28515625" style="23" customWidth="1"/>
-    <col min="7" max="7" width="13.42578125" style="23" customWidth="1"/>
+    <col min="2" max="2" width="40.109375" style="23" customWidth="1"/>
+    <col min="3" max="3" width="10.33203125" style="23"/>
+    <col min="4" max="4" width="10.33203125" style="23" customWidth="1"/>
+    <col min="5" max="5" width="13.5546875" style="23" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" style="23" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" style="23" customWidth="1"/>
     <col min="8" max="8" width="3" style="23" customWidth="1"/>
-    <col min="9" max="13" width="10.7109375" style="23" customWidth="1"/>
-    <col min="14" max="16384" width="10.28515625" style="23"/>
+    <col min="9" max="13" width="10.6640625" style="23" customWidth="1"/>
+    <col min="14" max="16384" width="10.33203125" style="23"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="105"/>
       <c r="B1" s="106"/>
       <c r="C1" s="106"/>
@@ -8139,32 +8138,32 @@
       <c r="L1" s="106"/>
       <c r="M1" s="107"/>
     </row>
-    <row r="2" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="108"/>
-      <c r="B2" s="438" t="s">
+      <c r="B2" s="437" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="439"/>
-      <c r="D2" s="439"/>
-      <c r="E2" s="439"/>
-      <c r="F2" s="439"/>
-      <c r="G2" s="440"/>
+      <c r="C2" s="438"/>
+      <c r="D2" s="438"/>
+      <c r="E2" s="438"/>
+      <c r="F2" s="438"/>
+      <c r="G2" s="439"/>
       <c r="M2" s="109"/>
     </row>
-    <row r="3" spans="1:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="8.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="108"/>
       <c r="M3" s="109"/>
     </row>
-    <row r="4" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="108"/>
-      <c r="B4" s="450" t="s">
+      <c r="B4" s="449" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="450"/>
-      <c r="D4" s="450"/>
-      <c r="E4" s="450"/>
-      <c r="F4" s="450"/>
-      <c r="G4" s="450"/>
+      <c r="C4" s="449"/>
+      <c r="D4" s="449"/>
+      <c r="E4" s="449"/>
+      <c r="F4" s="449"/>
+      <c r="G4" s="449"/>
       <c r="H4" s="104"/>
       <c r="I4" s="104"/>
       <c r="J4" s="104"/>
@@ -8175,16 +8174,16 @@
       <c r="O4" s="104"/>
       <c r="P4" s="104"/>
     </row>
-    <row r="5" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="108"/>
-      <c r="B5" s="450" t="s">
+      <c r="B5" s="449" t="s">
         <v>161</v>
       </c>
-      <c r="C5" s="450"/>
-      <c r="D5" s="450"/>
-      <c r="E5" s="450"/>
-      <c r="F5" s="450"/>
-      <c r="G5" s="450"/>
+      <c r="C5" s="449"/>
+      <c r="D5" s="449"/>
+      <c r="E5" s="449"/>
+      <c r="F5" s="449"/>
+      <c r="G5" s="449"/>
       <c r="H5" s="104"/>
       <c r="I5" s="104"/>
       <c r="J5" s="104"/>
@@ -8195,11 +8194,11 @@
       <c r="O5" s="104"/>
       <c r="P5" s="104"/>
     </row>
-    <row r="6" spans="1:16" ht="5.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="108"/>
       <c r="M6" s="109"/>
     </row>
-    <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="108"/>
       <c r="B7" s="183" t="s">
         <v>40</v>
@@ -8213,7 +8212,7 @@
       </c>
       <c r="M7" s="109"/>
     </row>
-    <row r="8" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="108"/>
       <c r="B8" s="184" t="s">
         <v>41</v>
@@ -8229,7 +8228,7 @@
       </c>
       <c r="M8" s="109"/>
     </row>
-    <row r="9" spans="1:16" ht="17.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="108"/>
       <c r="B9" s="184" t="s">
         <v>42</v>
@@ -8242,7 +8241,7 @@
       <c r="G9" s="84"/>
       <c r="M9" s="109"/>
     </row>
-    <row r="10" spans="1:16" ht="15.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="15.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="108"/>
       <c r="B10" s="184" t="s">
         <v>43</v>
@@ -8255,7 +8254,7 @@
       <c r="G10" s="84"/>
       <c r="M10" s="109"/>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" s="108"/>
       <c r="B11" s="185" t="s">
         <v>44</v>
@@ -8270,13 +8269,13 @@
       <c r="G11" s="30"/>
       <c r="M11" s="109"/>
     </row>
-    <row r="12" spans="1:16" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="108"/>
       <c r="C12" s="73"/>
       <c r="D12" s="73"/>
       <c r="M12" s="109"/>
     </row>
-    <row r="13" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="223">
         <v>1</v>
       </c>
@@ -8289,7 +8288,7 @@
       <c r="D13" s="186">
         <v>1</v>
       </c>
-      <c r="E13" s="449" t="s">
+      <c r="E13" s="448" t="s">
         <v>45</v>
       </c>
       <c r="F13" s="232" t="s">
@@ -8300,7 +8299,7 @@
       <c r="I13" s="234"/>
       <c r="M13" s="109"/>
     </row>
-    <row r="14" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="223">
         <v>2</v>
       </c>
@@ -8314,7 +8313,7 @@
         <f>+FORMATO!G20</f>
         <v>0</v>
       </c>
-      <c r="E14" s="449"/>
+      <c r="E14" s="448"/>
       <c r="F14" s="235" t="s">
         <v>154</v>
       </c>
@@ -8325,7 +8324,7 @@
       </c>
       <c r="M14" s="109"/>
     </row>
-    <row r="15" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="223">
         <v>3</v>
       </c>
@@ -8353,7 +8352,7 @@
       </c>
       <c r="M15" s="109"/>
     </row>
-    <row r="16" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:16" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="223">
         <v>4</v>
       </c>
@@ -8375,7 +8374,7 @@
       <c r="G16" s="226"/>
       <c r="M16" s="109"/>
     </row>
-    <row r="17" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="223">
         <v>5</v>
       </c>
@@ -8397,7 +8396,7 @@
       <c r="G17" s="226"/>
       <c r="M17" s="109"/>
     </row>
-    <row r="18" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="223">
         <v>6</v>
       </c>
@@ -8419,7 +8418,7 @@
       <c r="G18" s="226"/>
       <c r="M18" s="109"/>
     </row>
-    <row r="19" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="223">
         <v>7</v>
       </c>
@@ -8441,7 +8440,7 @@
       <c r="G19" s="228"/>
       <c r="M19" s="109"/>
     </row>
-    <row r="20" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="223">
         <v>8</v>
       </c>
@@ -8463,7 +8462,7 @@
       <c r="G20" s="228"/>
       <c r="M20" s="109"/>
     </row>
-    <row r="21" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="223">
         <v>9</v>
       </c>
@@ -8485,7 +8484,7 @@
       <c r="G21" s="228"/>
       <c r="M21" s="109"/>
     </row>
-    <row r="22" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="108"/>
       <c r="B22" s="35"/>
       <c r="C22" s="35"/>
@@ -8495,7 +8494,7 @@
       </c>
       <c r="M22" s="109"/>
     </row>
-    <row r="23" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="108"/>
       <c r="B23" s="88" t="s">
         <v>49</v>
@@ -8513,7 +8512,7 @@
       <c r="G23" s="230"/>
       <c r="M23" s="109"/>
     </row>
-    <row r="24" spans="1:13" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" ht="10.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="108"/>
       <c r="B24" s="35"/>
       <c r="C24" s="35"/>
@@ -8521,29 +8520,29 @@
       <c r="E24" s="35"/>
       <c r="M24" s="109"/>
     </row>
-    <row r="25" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="108"/>
-      <c r="B25" s="441" t="s">
+      <c r="B25" s="440" t="s">
         <v>148</v>
       </c>
-      <c r="C25" s="442"/>
-      <c r="D25" s="445" t="s">
+      <c r="C25" s="441"/>
+      <c r="D25" s="444" t="s">
         <v>50</v>
       </c>
-      <c r="E25" s="447" t="s">
+      <c r="E25" s="446" t="s">
         <v>51</v>
       </c>
       <c r="M25" s="109"/>
     </row>
-    <row r="26" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="108"/>
-      <c r="B26" s="443"/>
-      <c r="C26" s="444"/>
-      <c r="D26" s="446"/>
-      <c r="E26" s="448"/>
+      <c r="B26" s="442"/>
+      <c r="C26" s="443"/>
+      <c r="D26" s="445"/>
+      <c r="E26" s="447"/>
       <c r="M26" s="109"/>
     </row>
-    <row r="27" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="108"/>
       <c r="B27" s="214" t="s">
         <v>52</v>
@@ -8557,9 +8556,9 @@
       <c r="E27" s="192"/>
       <c r="M27" s="109"/>
     </row>
-    <row r="28" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="108"/>
-      <c r="B28" s="437" t="s">
+      <c r="B28" s="436" t="s">
         <v>54</v>
       </c>
       <c r="C28" s="93" t="s">
@@ -8571,9 +8570,9 @@
       <c r="E28" s="193"/>
       <c r="M28" s="109"/>
     </row>
-    <row r="29" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="108"/>
-      <c r="B29" s="437"/>
+      <c r="B29" s="436"/>
       <c r="C29" s="93" t="s">
         <v>137</v>
       </c>
@@ -8583,9 +8582,9 @@
       <c r="E29" s="193"/>
       <c r="M29" s="109"/>
     </row>
-    <row r="30" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="108"/>
-      <c r="B30" s="437"/>
+      <c r="B30" s="436"/>
       <c r="C30" s="93" t="s">
         <v>138</v>
       </c>
@@ -8595,9 +8594,9 @@
       <c r="E30" s="193"/>
       <c r="M30" s="109"/>
     </row>
-    <row r="31" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="108"/>
-      <c r="B31" s="437"/>
+      <c r="B31" s="436"/>
       <c r="C31" s="93" t="s">
         <v>139</v>
       </c>
@@ -8607,9 +8606,9 @@
       <c r="E31" s="193"/>
       <c r="M31" s="109"/>
     </row>
-    <row r="32" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="108"/>
-      <c r="B32" s="437"/>
+      <c r="B32" s="436"/>
       <c r="C32" s="93" t="s">
         <v>140</v>
       </c>
@@ -8619,9 +8618,9 @@
       <c r="E32" s="194"/>
       <c r="M32" s="109"/>
     </row>
-    <row r="33" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="108"/>
-      <c r="B33" s="437"/>
+      <c r="B33" s="436"/>
       <c r="C33" s="95" t="s">
         <v>141</v>
       </c>
@@ -8631,9 +8630,9 @@
       <c r="E33" s="195"/>
       <c r="M33" s="109"/>
     </row>
-    <row r="34" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="108"/>
-      <c r="B34" s="437"/>
+      <c r="B34" s="436"/>
       <c r="C34" s="178" t="s">
         <v>142</v>
       </c>
@@ -8643,9 +8642,9 @@
       <c r="E34" s="195"/>
       <c r="M34" s="109"/>
     </row>
-    <row r="35" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="108"/>
-      <c r="B35" s="437"/>
+      <c r="B35" s="436"/>
       <c r="C35" s="95" t="s">
         <v>143</v>
       </c>
@@ -8655,9 +8654,9 @@
       <c r="E35" s="195"/>
       <c r="M35" s="109"/>
     </row>
-    <row r="36" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="108"/>
-      <c r="B36" s="437"/>
+      <c r="B36" s="436"/>
       <c r="C36" s="96" t="s">
         <v>144</v>
       </c>
@@ -8667,9 +8666,9 @@
       <c r="E36" s="195"/>
       <c r="M36" s="109"/>
     </row>
-    <row r="37" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="108"/>
-      <c r="B37" s="437"/>
+      <c r="B37" s="436"/>
       <c r="C37" s="95" t="s">
         <v>145</v>
       </c>
@@ -8679,9 +8678,9 @@
       <c r="E37" s="195"/>
       <c r="M37" s="109"/>
     </row>
-    <row r="38" spans="1:13" ht="13.9" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="108"/>
-      <c r="B38" s="437"/>
+      <c r="B38" s="436"/>
       <c r="C38" s="95" t="s">
         <v>146</v>
       </c>
@@ -8691,7 +8690,7 @@
       <c r="E38" s="195"/>
       <c r="M38" s="109"/>
     </row>
-    <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="111"/>
       <c r="B39" s="86"/>
       <c r="C39" s="77"/>
@@ -8704,7 +8703,7 @@
       </c>
       <c r="M39" s="109"/>
     </row>
-    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="111"/>
       <c r="B40" s="86"/>
       <c r="C40" s="77"/>
@@ -8717,7 +8716,7 @@
       </c>
       <c r="M40" s="109"/>
     </row>
-    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="111"/>
       <c r="B41" s="86"/>
       <c r="C41" s="99"/>
@@ -8730,7 +8729,7 @@
       </c>
       <c r="M41" s="109"/>
     </row>
-    <row r="42" spans="1:13" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" ht="5.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="112"/>
       <c r="B42" s="113"/>
       <c r="C42" s="113"/>
@@ -8775,26 +8774,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M61"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.42578125" style="13" customWidth="1"/>
-    <col min="2" max="8" width="14.140625" style="13" customWidth="1"/>
-    <col min="9" max="9" width="9.85546875" style="13" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" style="13" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="13"/>
+    <col min="1" max="1" width="22.44140625" style="13" customWidth="1"/>
+    <col min="2" max="8" width="14.109375" style="13" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" style="13" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" style="13" customWidth="1"/>
+    <col min="11" max="16384" width="11.44140625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="459"/>
-      <c r="B1" s="460"/>
-      <c r="C1" s="465" t="s">
+    <row r="1" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="450"/>
+      <c r="B1" s="451"/>
+      <c r="C1" s="456" t="s">
         <v>57</v>
       </c>
-      <c r="D1" s="466"/>
-      <c r="E1" s="466"/>
-      <c r="F1" s="466"/>
-      <c r="G1" s="466"/>
-      <c r="H1" s="467"/>
+      <c r="D1" s="457"/>
+      <c r="E1" s="457"/>
+      <c r="F1" s="457"/>
+      <c r="G1" s="457"/>
+      <c r="H1" s="458"/>
       <c r="I1" s="117" t="s">
         <v>58</v>
       </c>
@@ -8802,15 +8801,15 @@
         <v>59</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="461"/>
-      <c r="B2" s="462"/>
-      <c r="C2" s="468"/>
-      <c r="D2" s="469"/>
-      <c r="E2" s="469"/>
-      <c r="F2" s="469"/>
-      <c r="G2" s="469"/>
-      <c r="H2" s="470"/>
+    <row r="2" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="452"/>
+      <c r="B2" s="453"/>
+      <c r="C2" s="459"/>
+      <c r="D2" s="460"/>
+      <c r="E2" s="460"/>
+      <c r="F2" s="460"/>
+      <c r="G2" s="460"/>
+      <c r="H2" s="461"/>
       <c r="I2" s="117" t="s">
         <v>60</v>
       </c>
@@ -8818,15 +8817,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="461"/>
-      <c r="B3" s="462"/>
-      <c r="C3" s="468"/>
-      <c r="D3" s="469"/>
-      <c r="E3" s="469"/>
-      <c r="F3" s="469"/>
-      <c r="G3" s="469"/>
-      <c r="H3" s="470"/>
+    <row r="3" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="452"/>
+      <c r="B3" s="453"/>
+      <c r="C3" s="459"/>
+      <c r="D3" s="460"/>
+      <c r="E3" s="460"/>
+      <c r="F3" s="460"/>
+      <c r="G3" s="460"/>
+      <c r="H3" s="461"/>
       <c r="I3" s="117" t="s">
         <v>61</v>
       </c>
@@ -8834,15 +8833,15 @@
         <v>46146</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="463"/>
-      <c r="B4" s="464"/>
-      <c r="C4" s="471"/>
-      <c r="D4" s="472"/>
-      <c r="E4" s="472"/>
-      <c r="F4" s="472"/>
-      <c r="G4" s="472"/>
-      <c r="H4" s="473"/>
+    <row r="4" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="454"/>
+      <c r="B4" s="455"/>
+      <c r="C4" s="462"/>
+      <c r="D4" s="463"/>
+      <c r="E4" s="463"/>
+      <c r="F4" s="463"/>
+      <c r="G4" s="463"/>
+      <c r="H4" s="464"/>
       <c r="I4" s="117" t="s">
         <v>62</v>
       </c>
@@ -8850,7 +8849,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="119" t="s">
         <v>64</v>
       </c>
@@ -8866,7 +8865,7 @@
       <c r="I6" s="15"/>
       <c r="J6" s="14"/>
     </row>
-    <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="119" t="s">
         <v>65</v>
       </c>
@@ -8882,7 +8881,7 @@
       <c r="I7" s="15"/>
       <c r="J7" s="14"/>
     </row>
-    <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="119" t="s">
         <v>66</v>
       </c>
@@ -8898,7 +8897,7 @@
       <c r="I8" s="15"/>
       <c r="J8" s="14"/>
     </row>
-    <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="120" t="s">
         <v>68</v>
       </c>
@@ -8915,8 +8914,8 @@
       <c r="J9" s="14"/>
       <c r="M9" s="221"/>
     </row>
-    <row r="10" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="11" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="134" t="s">
         <v>70</v>
       </c>
@@ -8931,7 +8930,7 @@
       <c r="J11" s="18"/>
       <c r="K11" s="18"/>
     </row>
-    <row r="12" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="18"/>
       <c r="B12" s="18"/>
       <c r="C12" s="18"/>
@@ -8944,7 +8943,7 @@
       <c r="J12" s="18"/>
       <c r="K12" s="18"/>
     </row>
-    <row r="13" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="219" t="s">
         <v>71</v>
       </c>
@@ -8961,7 +8960,7 @@
       <c r="J13" s="18"/>
       <c r="K13" s="18"/>
     </row>
-    <row r="14" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="18"/>
       <c r="B14" s="18"/>
       <c r="C14" s="18"/>
@@ -8974,7 +8973,7 @@
       <c r="J14" s="18"/>
       <c r="K14" s="18"/>
     </row>
-    <row r="15" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="220" t="s">
         <v>72</v>
       </c>
@@ -8989,7 +8988,7 @@
       <c r="J15" s="18"/>
       <c r="K15" s="18"/>
     </row>
-    <row r="16" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="220" t="s">
         <v>73</v>
       </c>
@@ -9004,7 +9003,7 @@
       <c r="J16" s="18"/>
       <c r="K16" s="18"/>
     </row>
-    <row r="17" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="18"/>
       <c r="B17" s="18"/>
       <c r="C17" s="18"/>
@@ -9017,7 +9016,7 @@
       <c r="J17" s="18"/>
       <c r="K17" s="18"/>
     </row>
-    <row r="18" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="219" t="s">
         <v>75</v>
       </c>
@@ -9032,7 +9031,7 @@
       <c r="J18" s="18"/>
       <c r="K18" s="18"/>
     </row>
-    <row r="19" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="18"/>
       <c r="B19" s="18"/>
       <c r="C19" s="18"/>
@@ -9045,7 +9044,7 @@
       <c r="J19" s="18"/>
       <c r="K19" s="18"/>
     </row>
-    <row r="20" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="220" t="s">
         <v>76</v>
       </c>
@@ -9060,7 +9059,7 @@
       <c r="J20" s="18"/>
       <c r="K20" s="18"/>
     </row>
-    <row r="21" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="18"/>
       <c r="B21" s="18"/>
       <c r="C21" s="18"/>
@@ -9073,7 +9072,7 @@
       <c r="J21" s="18"/>
       <c r="K21" s="18"/>
     </row>
-    <row r="22" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="134" t="s">
         <v>77</v>
       </c>
@@ -9088,7 +9087,7 @@
       <c r="J22" s="18"/>
       <c r="K22" s="18"/>
     </row>
-    <row r="23" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="18"/>
       <c r="B23" s="18"/>
       <c r="C23" s="18"/>
@@ -9101,7 +9100,7 @@
       <c r="J23" s="18"/>
       <c r="K23" s="18"/>
     </row>
-    <row r="24" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="18"/>
       <c r="B24" s="18"/>
       <c r="C24" s="18"/>
@@ -9114,7 +9113,7 @@
       <c r="J24" s="18"/>
       <c r="K24" s="18"/>
     </row>
-    <row r="25" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="18"/>
       <c r="B25" s="18"/>
       <c r="C25" s="18"/>
@@ -9127,7 +9126,7 @@
       <c r="J25" s="18"/>
       <c r="K25" s="18"/>
     </row>
-    <row r="26" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="18"/>
       <c r="B26" s="18"/>
       <c r="C26" s="18"/>
@@ -9140,7 +9139,7 @@
       <c r="J26" s="18"/>
       <c r="K26" s="19"/>
     </row>
-    <row r="27" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="18"/>
       <c r="B27" s="18"/>
       <c r="C27" s="18"/>
@@ -9153,7 +9152,7 @@
       <c r="J27" s="18"/>
       <c r="K27" s="18"/>
     </row>
-    <row r="28" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="18"/>
       <c r="B28" s="18"/>
       <c r="C28" s="18"/>
@@ -9166,7 +9165,7 @@
       <c r="J28" s="18"/>
       <c r="K28" s="18"/>
     </row>
-    <row r="29" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="18"/>
       <c r="B29" s="18"/>
       <c r="C29" s="18"/>
@@ -9179,7 +9178,7 @@
       <c r="J29" s="18"/>
       <c r="K29" s="18"/>
     </row>
-    <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="18"/>
       <c r="B30" s="18"/>
       <c r="C30" s="18"/>
@@ -9192,7 +9191,7 @@
       <c r="J30" s="18"/>
       <c r="K30" s="18"/>
     </row>
-    <row r="31" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="18"/>
       <c r="B31" s="18"/>
       <c r="C31" s="18"/>
@@ -9205,7 +9204,7 @@
       <c r="J31" s="18"/>
       <c r="K31" s="18"/>
     </row>
-    <row r="32" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="18"/>
       <c r="B32" s="18"/>
       <c r="C32" s="18"/>
@@ -9218,7 +9217,7 @@
       <c r="J32" s="18"/>
       <c r="K32" s="18"/>
     </row>
-    <row r="33" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="18"/>
       <c r="B33" s="18"/>
       <c r="C33" s="18"/>
@@ -9231,7 +9230,7 @@
       <c r="J33" s="18"/>
       <c r="K33" s="18"/>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A34" s="18"/>
       <c r="B34" s="18"/>
       <c r="C34" s="18"/>
@@ -9244,25 +9243,25 @@
       <c r="J34" s="18"/>
       <c r="K34" s="18"/>
     </row>
-    <row r="35" spans="1:12" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:12" ht="10.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="I35" s="125"/>
       <c r="J35" s="125"/>
     </row>
-    <row r="36" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="476" t="s">
+    <row r="36" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="467" t="s">
         <v>78</v>
       </c>
-      <c r="B36" s="477"/>
-      <c r="C36" s="477"/>
-      <c r="D36" s="477"/>
-      <c r="E36" s="477"/>
-      <c r="F36" s="477"/>
-      <c r="G36" s="477"/>
-      <c r="H36" s="478"/>
+      <c r="B36" s="468"/>
+      <c r="C36" s="468"/>
+      <c r="D36" s="468"/>
+      <c r="E36" s="468"/>
+      <c r="F36" s="468"/>
+      <c r="G36" s="468"/>
+      <c r="H36" s="469"/>
       <c r="I36" s="125"/>
       <c r="J36" s="125"/>
     </row>
-    <row r="37" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="204" t="s">
         <v>79</v>
       </c>
@@ -9290,7 +9289,7 @@
       <c r="I37" s="125"/>
       <c r="J37" s="125"/>
     </row>
-    <row r="38" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="199" t="s">
         <v>87</v>
       </c>
@@ -9321,7 +9320,7 @@
       <c r="K38" s="13"/>
       <c r="L38" s="13"/>
     </row>
-    <row r="39" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="153" t="s">
         <v>89</v>
       </c>
@@ -9357,7 +9356,7 @@
       <c r="K39" s="13"/>
       <c r="L39" s="13"/>
     </row>
-    <row r="40" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="139" t="s">
         <v>90</v>
       </c>
@@ -9387,7 +9386,7 @@
       <c r="K40" s="13"/>
       <c r="L40" s="13"/>
     </row>
-    <row r="41" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="139" t="s">
         <v>92</v>
       </c>
@@ -9417,7 +9416,7 @@
       <c r="K41" s="13"/>
       <c r="L41" s="13"/>
     </row>
-    <row r="42" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="139" t="s">
         <v>94</v>
       </c>
@@ -9447,7 +9446,7 @@
       <c r="K42" s="13"/>
       <c r="L42" s="13"/>
     </row>
-    <row r="43" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="147" t="s">
         <v>96</v>
       </c>
@@ -9481,7 +9480,7 @@
       <c r="K43" s="13"/>
       <c r="L43" s="13"/>
     </row>
-    <row r="44" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="139" t="s">
         <v>90</v>
       </c>
@@ -9511,7 +9510,7 @@
       <c r="K44" s="13"/>
       <c r="L44" s="13"/>
     </row>
-    <row r="45" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="139" t="s">
         <v>92</v>
       </c>
@@ -9541,7 +9540,7 @@
       <c r="K45" s="13"/>
       <c r="L45" s="13"/>
     </row>
-    <row r="46" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="139" t="s">
         <v>94</v>
       </c>
@@ -9601,44 +9600,44 @@
       <c r="J47" s="125"/>
     </row>
     <row r="48" spans="1:12" s="122" customFormat="1" ht="24.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="481" t="s">
+      <c r="A48" s="472" t="s">
         <v>99</v>
       </c>
-      <c r="B48" s="482"/>
-      <c r="C48" s="482"/>
-      <c r="D48" s="482"/>
+      <c r="B48" s="473"/>
+      <c r="C48" s="473"/>
+      <c r="D48" s="473"/>
       <c r="E48" s="215" t="s">
         <v>32</v>
       </c>
-      <c r="F48" s="479" t="e">
+      <c r="F48" s="470" t="e">
         <f>SQRT((H39*H39)+(H43*H43)+(H47*H47))</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G48" s="479"/>
-      <c r="H48" s="480"/>
+      <c r="G48" s="470"/>
+      <c r="H48" s="471"/>
       <c r="I48" s="125"/>
       <c r="J48" s="125"/>
     </row>
     <row r="49" spans="1:10" s="122" customFormat="1" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="483" t="s">
+      <c r="A49" s="474" t="s">
         <v>100</v>
       </c>
-      <c r="B49" s="484"/>
-      <c r="C49" s="484"/>
-      <c r="D49" s="484"/>
+      <c r="B49" s="475"/>
+      <c r="C49" s="475"/>
+      <c r="D49" s="475"/>
       <c r="E49" s="146" t="s">
         <v>32</v>
       </c>
-      <c r="F49" s="474" t="e">
+      <c r="F49" s="465" t="e">
         <f>F48*2</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="G49" s="474"/>
-      <c r="H49" s="475"/>
+      <c r="G49" s="465"/>
+      <c r="H49" s="466"/>
       <c r="I49" s="125"/>
       <c r="J49" s="125"/>
     </row>
-    <row r="50" spans="1:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="125"/>
       <c r="D50" s="125"/>
       <c r="E50" s="125"/>
@@ -9648,7 +9647,7 @@
       <c r="I50" s="125"/>
       <c r="J50" s="125"/>
     </row>
-    <row r="51" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="127"/>
       <c r="B51" s="128" t="s">
         <v>101</v>
@@ -9666,7 +9665,7 @@
       <c r="I51" s="125"/>
       <c r="J51" s="125"/>
     </row>
-    <row r="52" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="123"/>
       <c r="B52" s="124" t="str">
         <f>A39</f>
@@ -9687,7 +9686,7 @@
       <c r="I52" s="125"/>
       <c r="J52" s="125"/>
     </row>
-    <row r="53" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="123"/>
       <c r="B53" s="124" t="str">
         <f>A43</f>
@@ -9708,7 +9707,7 @@
       <c r="I53" s="125"/>
       <c r="J53" s="125"/>
     </row>
-    <row r="54" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="123"/>
       <c r="B54" s="124" t="str">
         <f>A47</f>
@@ -9729,7 +9728,7 @@
       <c r="I54" s="125"/>
       <c r="J54" s="125"/>
     </row>
-    <row r="55" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="125"/>
       <c r="C55" s="132" t="e">
         <f>SUM(C52:C54)</f>
@@ -9746,7 +9745,7 @@
       <c r="I55" s="125"/>
       <c r="J55" s="125"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="125"/>
       <c r="B56" s="125"/>
       <c r="C56" s="125"/>
@@ -9758,7 +9757,7 @@
       <c r="I56" s="125"/>
       <c r="J56" s="125"/>
     </row>
-    <row r="57" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="125"/>
       <c r="E57" s="125"/>
       <c r="F57" s="125"/>
@@ -9767,7 +9766,7 @@
       <c r="I57" s="125"/>
       <c r="J57" s="125"/>
     </row>
-    <row r="58" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="125"/>
       <c r="E58" s="125"/>
       <c r="F58" s="125"/>
@@ -9776,25 +9775,25 @@
       <c r="I58" s="125"/>
       <c r="J58" s="125"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="385" t="s">
         <v>202</v>
       </c>
-      <c r="B59" s="451" t="s">
+      <c r="B59" s="476" t="s">
         <v>203</v>
       </c>
-      <c r="C59" s="452"/>
+      <c r="C59" s="477"/>
       <c r="D59" s="386"/>
-      <c r="E59" s="453" t="s">
+      <c r="E59" s="478" t="s">
         <v>204</v>
       </c>
-      <c r="F59" s="453"/>
-      <c r="G59" s="454" t="s">
+      <c r="F59" s="478"/>
+      <c r="G59" s="479" t="s">
         <v>205</v>
       </c>
-      <c r="H59" s="455"/>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="H59" s="480"/>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="243"/>
       <c r="B60" s="243"/>
       <c r="C60" s="243"/>
@@ -9804,27 +9803,33 @@
       <c r="G60" s="243"/>
       <c r="H60" s="243"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="387" t="s">
         <v>206</v>
       </c>
-      <c r="B61" s="456">
+      <c r="B61" s="481">
         <v>44869</v>
       </c>
-      <c r="C61" s="457"/>
+      <c r="C61" s="482"/>
       <c r="D61" s="243"/>
-      <c r="E61" s="458" t="s">
+      <c r="E61" s="483" t="s">
         <v>207</v>
       </c>
-      <c r="F61" s="458"/>
-      <c r="G61" s="456">
+      <c r="F61" s="483"/>
+      <c r="G61" s="481">
         <v>44870</v>
       </c>
-      <c r="H61" s="457"/>
+      <c r="H61" s="482"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="E4saOIWIh+Eme1oJwQuMKDkpQOD3mu/gNSXXqxi1z9FTNqSBh3K6FNpoNItb60yc5uGoFN6+zjqUl8BeksL6fA==" saltValue="903QStExJ+2hr453WB5skg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="13">
+    <mergeCell ref="B59:C59"/>
+    <mergeCell ref="E59:F59"/>
+    <mergeCell ref="G59:H59"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="G61:H61"/>
     <mergeCell ref="A1:B4"/>
     <mergeCell ref="C1:H4"/>
     <mergeCell ref="F49:H49"/>
@@ -9832,12 +9837,6 @@
     <mergeCell ref="F48:H48"/>
     <mergeCell ref="A48:D48"/>
     <mergeCell ref="A49:D49"/>
-    <mergeCell ref="B59:C59"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="G59:H59"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="G61:H61"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.31496062992125984" top="0.74803149606299213" bottom="0.55118110236220474" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="70" orientation="portrait" r:id="rId1"/>
@@ -9848,31 +9847,31 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:P31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.28515625" style="240" customWidth="1"/>
+    <col min="1" max="1" width="4.33203125" style="240" customWidth="1"/>
     <col min="2" max="2" width="12" style="240" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" style="240" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" style="240" customWidth="1"/>
     <col min="4" max="4" width="12" style="240" customWidth="1"/>
-    <col min="5" max="7" width="11.42578125" style="240"/>
-    <col min="8" max="8" width="14.42578125" style="240" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="240"/>
-    <col min="10" max="10" width="11.85546875" style="240" customWidth="1"/>
-    <col min="11" max="16384" width="11.42578125" style="240"/>
+    <col min="5" max="7" width="11.44140625" style="240"/>
+    <col min="8" max="8" width="14.44140625" style="240" customWidth="1"/>
+    <col min="9" max="9" width="11.44140625" style="240"/>
+    <col min="10" max="10" width="11.88671875" style="240" customWidth="1"/>
+    <col min="11" max="16384" width="11.44140625" style="240"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B1" s="485" t="s">
+    <row r="1" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B1" s="484" t="s">
         <v>103</v>
       </c>
-      <c r="C1" s="485"/>
-      <c r="D1" s="485"/>
-      <c r="E1" s="485"/>
-      <c r="F1" s="485"/>
-      <c r="G1" s="485"/>
-      <c r="H1" s="485"/>
-    </row>
-    <row r="2" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="C1" s="484"/>
+      <c r="D1" s="484"/>
+      <c r="E1" s="484"/>
+      <c r="F1" s="484"/>
+      <c r="G1" s="484"/>
+      <c r="H1" s="484"/>
+    </row>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B2" s="241"/>
       <c r="C2" s="242"/>
       <c r="D2" s="242"/>
@@ -9881,7 +9880,7 @@
       <c r="G2" s="243"/>
       <c r="H2" s="243"/>
     </row>
-    <row r="3" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B3" s="241"/>
       <c r="C3" s="242"/>
       <c r="D3" s="242"/>
@@ -9890,7 +9889,7 @@
       <c r="G3" s="243"/>
       <c r="H3" s="243"/>
     </row>
-    <row r="4" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B4" s="241"/>
       <c r="C4" s="242"/>
       <c r="D4" s="242"/>
@@ -9899,7 +9898,7 @@
       <c r="G4" s="243"/>
       <c r="H4" s="243"/>
     </row>
-    <row r="5" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="241"/>
       <c r="C5" s="242"/>
       <c r="D5" s="242"/>
@@ -9908,7 +9907,7 @@
       <c r="G5" s="243"/>
       <c r="H5" s="243"/>
     </row>
-    <row r="6" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="374" t="s">
         <v>192</v>
       </c>
@@ -9921,7 +9920,7 @@
       <c r="G6" s="243"/>
       <c r="H6" s="243"/>
     </row>
-    <row r="7" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="134" t="s">
         <v>104</v>
       </c>
@@ -9936,7 +9935,7 @@
       <c r="G7" s="243"/>
       <c r="H7" s="243"/>
     </row>
-    <row r="8" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="134" t="s">
         <v>193</v>
       </c>
@@ -9949,7 +9948,7 @@
       <c r="G8" s="243"/>
       <c r="H8" s="243"/>
     </row>
-    <row r="9" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="134" t="s">
         <v>94</v>
       </c>
@@ -9964,7 +9963,7 @@
       <c r="G9" s="243"/>
       <c r="H9" s="243"/>
     </row>
-    <row r="10" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="134" t="s">
         <v>195</v>
       </c>
@@ -9977,7 +9976,7 @@
       <c r="G10" s="243"/>
       <c r="H10" s="243"/>
     </row>
-    <row r="11" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="134" t="s">
         <v>197</v>
       </c>
@@ -9990,7 +9989,7 @@
       <c r="G11" s="243"/>
       <c r="H11" s="243"/>
     </row>
-    <row r="12" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:9" ht="6.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="246"/>
       <c r="C12" s="244"/>
       <c r="D12" s="243"/>
@@ -9999,7 +9998,7 @@
       <c r="G12" s="243"/>
       <c r="H12" s="243"/>
     </row>
-    <row r="13" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="249" t="s">
         <v>159</v>
       </c>
@@ -10023,7 +10022,7 @@
       </c>
       <c r="I13" s="249"/>
     </row>
-    <row r="14" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="250"/>
       <c r="C14" s="251"/>
       <c r="D14" s="263"/>
@@ -10033,7 +10032,7 @@
       <c r="H14" s="263"/>
       <c r="I14" s="252"/>
     </row>
-    <row r="15" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="250"/>
       <c r="C15" s="251"/>
       <c r="D15" s="263"/>
@@ -10043,7 +10042,7 @@
       <c r="H15" s="263"/>
       <c r="I15" s="252"/>
     </row>
-    <row r="16" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B16" s="243"/>
       <c r="C16" s="243"/>
       <c r="D16" s="243"/>
@@ -10053,7 +10052,7 @@
       <c r="H16" s="243"/>
       <c r="I16" s="243"/>
     </row>
-    <row r="17" spans="2:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:16" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="253"/>
       <c r="C17" s="247" t="s">
         <v>106</v>
@@ -10075,23 +10074,23 @@
       </c>
       <c r="I17" s="254"/>
     </row>
-    <row r="19" spans="2:16" x14ac:dyDescent="0.2">
-      <c r="B19" s="486" t="s">
+    <row r="19" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="B19" s="485" t="s">
         <v>107</v>
       </c>
-      <c r="C19" s="486"/>
-      <c r="D19" s="486"/>
-      <c r="E19" s="486"/>
-      <c r="F19" s="486"/>
-      <c r="G19" s="486"/>
-      <c r="H19" s="486"/>
-      <c r="I19" s="486"/>
+      <c r="C19" s="485"/>
+      <c r="D19" s="485"/>
+      <c r="E19" s="485"/>
+      <c r="F19" s="485"/>
+      <c r="G19" s="485"/>
+      <c r="H19" s="485"/>
+      <c r="I19" s="485"/>
       <c r="M19" s="243"/>
       <c r="N19" s="243"/>
       <c r="O19" s="243"/>
       <c r="P19" s="243"/>
     </row>
-    <row r="20" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B20" s="255"/>
       <c r="F20" s="243"/>
       <c r="I20" s="256"/>
@@ -10100,7 +10099,7 @@
       <c r="O20" s="243"/>
       <c r="P20" s="243"/>
     </row>
-    <row r="21" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="255"/>
       <c r="D21" s="249">
         <f>+D13</f>
@@ -10128,7 +10127,7 @@
       <c r="O21" s="243"/>
       <c r="P21" s="243"/>
     </row>
-    <row r="22" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B22" s="255"/>
       <c r="D22" s="217">
         <f>D17</f>
@@ -10156,7 +10155,7 @@
       <c r="O22" s="243"/>
       <c r="P22" s="243"/>
     </row>
-    <row r="23" spans="2:16" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B23" s="255"/>
       <c r="I23" s="257"/>
       <c r="M23" s="243"/>
@@ -10164,7 +10163,7 @@
       <c r="O23" s="243"/>
       <c r="P23" s="243"/>
     </row>
-    <row r="24" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="255"/>
       <c r="D24" s="138" t="s">
         <v>108</v>
@@ -10180,7 +10179,7 @@
       </c>
       <c r="I24" s="258"/>
     </row>
-    <row r="25" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="255"/>
       <c r="D25" s="138" t="s">
         <v>109</v>
@@ -10196,7 +10195,7 @@
       </c>
       <c r="I25" s="258"/>
     </row>
-    <row r="26" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="255"/>
       <c r="D26" s="138" t="s">
         <v>110</v>
@@ -10212,7 +10211,7 @@
       </c>
       <c r="I26" s="258"/>
     </row>
-    <row r="27" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="255"/>
       <c r="D27" s="138" t="s">
         <v>111</v>
@@ -10228,7 +10227,7 @@
       </c>
       <c r="I27" s="258"/>
     </row>
-    <row r="28" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="255"/>
       <c r="D28" s="138" t="s">
         <v>112</v>
@@ -10244,7 +10243,7 @@
       </c>
       <c r="I28" s="258"/>
     </row>
-    <row r="29" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B29" s="255"/>
       <c r="D29" s="121" t="s">
         <v>113</v>
@@ -10260,7 +10259,7 @@
       </c>
       <c r="I29" s="258"/>
     </row>
-    <row r="30" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="255"/>
       <c r="D30" s="121" t="s">
         <v>114</v>
@@ -10277,7 +10276,7 @@
       <c r="H30" s="259"/>
       <c r="I30" s="258"/>
     </row>
-    <row r="31" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:16" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="260"/>
       <c r="C31" s="261"/>
       <c r="D31" s="261"/>
@@ -10301,31 +10300,31 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B1:K8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.42578125" style="13" customWidth="1"/>
-    <col min="2" max="2" width="39.5703125" style="13" customWidth="1"/>
-    <col min="3" max="6" width="16.85546875" style="13" customWidth="1"/>
-    <col min="7" max="16384" width="11.42578125" style="13"/>
+    <col min="1" max="1" width="4.44140625" style="13" customWidth="1"/>
+    <col min="2" max="2" width="39.5546875" style="13" customWidth="1"/>
+    <col min="3" max="6" width="16.88671875" style="13" customWidth="1"/>
+    <col min="7" max="16384" width="11.44140625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="2" spans="2:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="488" t="s">
+    <row r="1" spans="2:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="487" t="s">
         <v>115</v>
       </c>
-      <c r="C2" s="489"/>
-      <c r="D2" s="489"/>
-      <c r="E2" s="489"/>
-      <c r="F2" s="490"/>
-    </row>
-    <row r="3" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="4" spans="2:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C2" s="488"/>
+      <c r="D2" s="488"/>
+      <c r="E2" s="488"/>
+      <c r="F2" s="489"/>
+    </row>
+    <row r="3" spans="2:11" ht="3.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="4" spans="2:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="158" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="5" spans="2:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="158" t="s">
         <v>117</v>
       </c>
@@ -10333,7 +10332,7 @@
         <v>46069</v>
       </c>
     </row>
-    <row r="6" spans="2:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="158" t="s">
         <v>118</v>
       </c>
@@ -10343,26 +10342,26 @@
       <c r="J6" s="116"/>
       <c r="K6" s="116"/>
     </row>
-    <row r="7" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="210" t="s">
         <v>119</v>
       </c>
-      <c r="C7" s="487">
+      <c r="C7" s="486">
         <v>0.1070306290533488</v>
       </c>
-      <c r="D7" s="487"/>
-      <c r="E7" s="487"/>
+      <c r="D7" s="486"/>
+      <c r="E7" s="486"/>
       <c r="F7" s="157"/>
     </row>
-    <row r="8" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="210" t="s">
         <v>120</v>
       </c>
-      <c r="C8" s="487">
+      <c r="C8" s="486">
         <v>0.11536174987114108</v>
       </c>
-      <c r="D8" s="487"/>
-      <c r="E8" s="487"/>
+      <c r="D8" s="486"/>
+      <c r="E8" s="486"/>
       <c r="F8" s="157"/>
     </row>
   </sheetData>
@@ -10380,22 +10379,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <sheetPr codeName="Hoja3"/>
   <dimension ref="A2:M9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="1" max="2" width="10.44140625" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="20" customWidth="1"/>
-    <col min="6" max="6" width="12.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" customWidth="1"/>
-    <col min="13" max="13" width="15.42578125" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" customWidth="1"/>
+    <col min="12" max="12" width="12.44140625" customWidth="1"/>
+    <col min="13" max="13" width="15.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="491" t="s">
+    <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="490" t="s">
         <v>121</v>
       </c>
-      <c r="B2" s="491"/>
+      <c r="B2" s="490"/>
       <c r="C2" s="5" t="s">
         <v>122</v>
       </c>
@@ -10430,7 +10429,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7">
         <v>4400</v>
       </c>
@@ -10476,7 +10475,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="6" t="str">
@@ -10513,7 +10512,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <f>+B3+1</f>
         <v>4402</v>
@@ -10556,7 +10555,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="1"/>
       <c r="C6" s="6" t="str">
@@ -10593,7 +10592,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <f>+B5+1</f>
         <v>4404</v>
@@ -10636,7 +10635,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="6" t="str">
@@ -10673,7 +10672,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:B2"/>

</xml_diff>